<commit_message>
fix: Correção dos dados tanto na leitura quanto na atualização dos dados
</commit_message>
<xml_diff>
--- a/DadosRomaneios.xlsx
+++ b/DadosRomaneios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.andrade\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01E987C0-B592-44A4-A9BC-66DDD4657C11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE11EF9-5BEB-4AF9-B4B3-109DCC56BD26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
   </bookViews>
@@ -4220,7 +4220,7 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" s="1">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="B89">
         <v>101</v>
@@ -4229,22 +4229,22 @@
         <v>46303</v>
       </c>
       <c r="D89" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="E89" t="s">
-        <v>73</v>
+        <v>12</v>
       </c>
       <c r="F89">
-        <v>69829</v>
+        <v>69306</v>
       </c>
       <c r="G89">
-        <v>178883</v>
+        <v>178885</v>
       </c>
       <c r="H89" s="2">
-        <v>8832</v>
+        <v>6579.82</v>
       </c>
       <c r="I89" s="1">
-        <v>46304</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.25">
@@ -4255,25 +4255,25 @@
         <v>101</v>
       </c>
       <c r="C90" s="1">
-        <v>46303</v>
+        <v>46293</v>
       </c>
       <c r="D90" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E90" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F90">
-        <v>69306</v>
+        <v>68061</v>
       </c>
       <c r="G90">
-        <v>178885</v>
+        <v>178140</v>
       </c>
       <c r="H90" s="2">
-        <v>6579.82</v>
+        <v>6791.6</v>
       </c>
       <c r="I90" s="1">
-        <v>46311</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.25">
@@ -4284,7 +4284,7 @@
         <v>101</v>
       </c>
       <c r="C91" s="1">
-        <v>46293</v>
+        <v>46301</v>
       </c>
       <c r="D91" t="s">
         <v>15</v>
@@ -4293,13 +4293,13 @@
         <v>16</v>
       </c>
       <c r="F91">
-        <v>68061</v>
+        <v>69133</v>
       </c>
       <c r="G91">
-        <v>178140</v>
+        <v>178759</v>
       </c>
       <c r="H91" s="2">
-        <v>6791.6</v>
+        <v>13819.85</v>
       </c>
       <c r="I91" s="1">
         <v>46294</v>
@@ -4313,7 +4313,7 @@
         <v>101</v>
       </c>
       <c r="C92" s="1">
-        <v>46301</v>
+        <v>46302</v>
       </c>
       <c r="D92" t="s">
         <v>15</v>
@@ -4322,13 +4322,13 @@
         <v>16</v>
       </c>
       <c r="F92">
-        <v>69133</v>
+        <v>68718</v>
       </c>
       <c r="G92">
-        <v>178759</v>
+        <v>178867</v>
       </c>
       <c r="H92" s="2">
-        <v>13819.85</v>
+        <v>8147.6</v>
       </c>
       <c r="I92" s="1">
         <v>46294</v>
@@ -4342,7 +4342,7 @@
         <v>101</v>
       </c>
       <c r="C93" s="1">
-        <v>46302</v>
+        <v>46292</v>
       </c>
       <c r="D93" t="s">
         <v>15</v>
@@ -4351,13 +4351,13 @@
         <v>16</v>
       </c>
       <c r="F93">
-        <v>68718</v>
+        <v>68717</v>
       </c>
       <c r="G93">
-        <v>178867</v>
+        <v>178106</v>
       </c>
       <c r="H93" s="2">
-        <v>8147.6</v>
+        <v>1645</v>
       </c>
       <c r="I93" s="1">
         <v>46294</v>
@@ -4371,7 +4371,7 @@
         <v>101</v>
       </c>
       <c r="C94" s="1">
-        <v>46292</v>
+        <v>46300</v>
       </c>
       <c r="D94" t="s">
         <v>15</v>
@@ -4380,13 +4380,13 @@
         <v>16</v>
       </c>
       <c r="F94">
-        <v>68717</v>
+        <v>67330</v>
       </c>
       <c r="G94">
-        <v>178106</v>
+        <v>178651</v>
       </c>
       <c r="H94" s="2">
-        <v>1645</v>
+        <v>467.6</v>
       </c>
       <c r="I94" s="1">
         <v>46294</v>
@@ -4400,22 +4400,22 @@
         <v>101</v>
       </c>
       <c r="C95" s="1">
-        <v>46300</v>
+        <v>46292</v>
       </c>
       <c r="D95" t="s">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="E95" t="s">
-        <v>16</v>
+        <v>75</v>
       </c>
       <c r="F95">
-        <v>67330</v>
+        <v>68527</v>
       </c>
       <c r="G95">
-        <v>178651</v>
+        <v>178089</v>
       </c>
       <c r="H95" s="2">
-        <v>467.6</v>
+        <v>591.27</v>
       </c>
       <c r="I95" s="1">
         <v>46294</v>
@@ -4429,22 +4429,22 @@
         <v>101</v>
       </c>
       <c r="C96" s="1">
-        <v>46292</v>
+        <v>46295</v>
       </c>
       <c r="D96" t="s">
-        <v>74</v>
+        <v>17</v>
       </c>
       <c r="E96" t="s">
-        <v>75</v>
+        <v>18</v>
       </c>
       <c r="F96">
-        <v>68527</v>
+        <v>67970</v>
       </c>
       <c r="G96">
-        <v>178089</v>
+        <v>178369</v>
       </c>
       <c r="H96" s="2">
-        <v>591.27</v>
+        <v>585.55999999999995</v>
       </c>
       <c r="I96" s="1">
         <v>46294</v>
@@ -4458,22 +4458,22 @@
         <v>101</v>
       </c>
       <c r="C97" s="1">
-        <v>46295</v>
+        <v>46302</v>
       </c>
       <c r="D97" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E97" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F97">
-        <v>67970</v>
+        <v>68410</v>
       </c>
       <c r="G97">
-        <v>178369</v>
+        <v>178868</v>
       </c>
       <c r="H97" s="2">
-        <v>585.55999999999995</v>
+        <v>7873.96</v>
       </c>
       <c r="I97" s="1">
         <v>46294</v>
@@ -4487,30 +4487,30 @@
         <v>101</v>
       </c>
       <c r="C98" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="D98" t="s">
-        <v>19</v>
+        <v>76</v>
       </c>
       <c r="E98" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="F98">
-        <v>68410</v>
+        <v>69685</v>
       </c>
       <c r="G98">
-        <v>178868</v>
+        <v>178871</v>
       </c>
       <c r="H98" s="2">
-        <v>7873.96</v>
+        <v>2569.75</v>
       </c>
       <c r="I98" s="1">
-        <v>46294</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B99">
         <v>101</v>
@@ -4519,22 +4519,22 @@
         <v>46303</v>
       </c>
       <c r="D99" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E99" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="F99">
-        <v>69685</v>
+        <v>69829</v>
       </c>
       <c r="G99">
-        <v>178871</v>
+        <v>178883</v>
       </c>
       <c r="H99" s="2">
-        <v>2569.75</v>
+        <v>8832</v>
       </c>
       <c r="I99" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
@@ -7652,7 +7652,7 @@
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A209" s="1">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B209">
         <v>101</v>
@@ -7661,27 +7661,27 @@
         <v>46304</v>
       </c>
       <c r="D209" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E209" t="s">
-        <v>165</v>
+        <v>1</v>
       </c>
       <c r="F209">
-        <v>68675</v>
+        <v>69149</v>
       </c>
       <c r="G209">
-        <v>179045</v>
+        <v>178999</v>
       </c>
       <c r="H209" s="2">
-        <v>2764.8</v>
+        <v>305.2</v>
       </c>
       <c r="I209" s="1">
-        <v>46304</v>
+        <v>46302</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A210" s="1">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B210">
         <v>101</v>
@@ -7690,22 +7690,22 @@
         <v>46304</v>
       </c>
       <c r="D210" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="E210" t="s">
-        <v>165</v>
+        <v>1</v>
       </c>
       <c r="F210">
-        <v>69744</v>
+        <v>69351</v>
       </c>
       <c r="G210">
-        <v>179044</v>
+        <v>179015</v>
       </c>
       <c r="H210" s="2">
-        <v>35025.4</v>
+        <v>2600.4499999999998</v>
       </c>
       <c r="I210" s="1">
-        <v>46304</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.25">
@@ -7725,16 +7725,16 @@
         <v>1</v>
       </c>
       <c r="F211">
-        <v>69149</v>
+        <v>69352</v>
       </c>
       <c r="G211">
-        <v>178999</v>
+        <v>178998</v>
       </c>
       <c r="H211" s="2">
-        <v>305.2</v>
+        <v>521.02</v>
       </c>
       <c r="I211" s="1">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.25">
@@ -7754,21 +7754,21 @@
         <v>1</v>
       </c>
       <c r="F212">
-        <v>69351</v>
+        <v>69437</v>
       </c>
       <c r="G212">
-        <v>179015</v>
+        <v>179039</v>
       </c>
       <c r="H212" s="2">
-        <v>2600.4499999999998</v>
+        <v>2078.34</v>
       </c>
       <c r="I212" s="1">
-        <v>46301</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A213" s="1">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B213">
         <v>101</v>
@@ -7777,27 +7777,27 @@
         <v>46304</v>
       </c>
       <c r="D213" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E213" t="s">
-        <v>1</v>
+        <v>165</v>
       </c>
       <c r="F213">
-        <v>69352</v>
+        <v>68675</v>
       </c>
       <c r="G213">
-        <v>178998</v>
+        <v>179045</v>
       </c>
       <c r="H213" s="2">
-        <v>521.02</v>
+        <v>2764.8</v>
       </c>
       <c r="I213" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A214" s="1">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B214">
         <v>101</v>
@@ -7806,22 +7806,22 @@
         <v>46304</v>
       </c>
       <c r="D214" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E214" t="s">
-        <v>1</v>
+        <v>165</v>
       </c>
       <c r="F214">
-        <v>69437</v>
+        <v>69744</v>
       </c>
       <c r="G214">
-        <v>179039</v>
+        <v>179044</v>
       </c>
       <c r="H214" s="2">
-        <v>2078.34</v>
+        <v>35025.4</v>
       </c>
       <c r="I214" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.25">
@@ -13491,80 +13491,86 @@
     </row>
     <row r="412" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A412" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B412">
         <v>101</v>
       </c>
       <c r="C412" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="D412" t="s">
-        <v>44</v>
+        <v>292</v>
       </c>
       <c r="E412" t="s">
-        <v>45</v>
+        <v>293</v>
+      </c>
+      <c r="F412">
+        <v>69392</v>
       </c>
       <c r="G412">
-        <v>179295</v>
+        <v>179006</v>
       </c>
       <c r="H412" s="2">
-        <v>15485.79</v>
+        <v>1983.9</v>
+      </c>
+      <c r="I412" s="1">
+        <v>46314</v>
       </c>
     </row>
     <row r="413" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A413" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B413">
         <v>101</v>
       </c>
       <c r="C413" s="1">
-        <v>46308</v>
+        <v>46304</v>
       </c>
       <c r="D413" t="s">
-        <v>44</v>
+        <v>294</v>
       </c>
       <c r="E413" t="s">
-        <v>45</v>
+        <v>295</v>
       </c>
       <c r="F413">
-        <v>69945</v>
+        <v>69310</v>
       </c>
       <c r="G413">
-        <v>179294</v>
+        <v>179035</v>
       </c>
       <c r="H413" s="2">
-        <v>2100</v>
+        <v>1271.0999999999999</v>
       </c>
       <c r="I413" s="1">
-        <v>46308</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="414" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A414" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B414">
         <v>101</v>
       </c>
       <c r="C414" s="1">
-        <v>46308</v>
+        <v>46305</v>
       </c>
       <c r="D414" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="E414" t="s">
-        <v>291</v>
+        <v>1</v>
       </c>
       <c r="F414">
-        <v>69656</v>
+        <v>69543</v>
       </c>
       <c r="G414">
-        <v>179270</v>
+        <v>179143</v>
       </c>
       <c r="H414" s="2">
-        <v>283.60000000000002</v>
+        <v>30712.720000000001</v>
       </c>
       <c r="I414" s="1">
         <v>46308</v>
@@ -13578,25 +13584,25 @@
         <v>101</v>
       </c>
       <c r="C415" s="1">
-        <v>46304</v>
+        <v>46306</v>
       </c>
       <c r="D415" t="s">
-        <v>292</v>
+        <v>11</v>
       </c>
       <c r="E415" t="s">
-        <v>293</v>
+        <v>12</v>
       </c>
       <c r="F415">
-        <v>69392</v>
+        <v>69343</v>
       </c>
       <c r="G415">
-        <v>179006</v>
+        <v>179180</v>
       </c>
       <c r="H415" s="2">
-        <v>1983.9</v>
+        <v>1281.22</v>
       </c>
       <c r="I415" s="1">
-        <v>46314</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="416" spans="1:9" x14ac:dyDescent="0.25">
@@ -13607,25 +13613,25 @@
         <v>101</v>
       </c>
       <c r="C416" s="1">
-        <v>46304</v>
+        <v>46307</v>
       </c>
       <c r="D416" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="E416" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F416">
-        <v>69310</v>
+        <v>69282</v>
       </c>
       <c r="G416">
-        <v>179035</v>
+        <v>179240</v>
       </c>
       <c r="H416" s="2">
-        <v>1271.0999999999999</v>
+        <v>6749.72</v>
       </c>
       <c r="I416" s="1">
-        <v>46311</v>
+        <v>46317</v>
       </c>
     </row>
     <row r="417" spans="1:9" x14ac:dyDescent="0.25">
@@ -13636,25 +13642,25 @@
         <v>101</v>
       </c>
       <c r="C417" s="1">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="D417" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="E417" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="F417">
-        <v>69543</v>
+        <v>67806</v>
       </c>
       <c r="G417">
-        <v>179143</v>
+        <v>179157</v>
       </c>
       <c r="H417" s="2">
-        <v>30712.720000000001</v>
+        <v>2556</v>
       </c>
       <c r="I417" s="1">
-        <v>46308</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="418" spans="1:9" x14ac:dyDescent="0.25">
@@ -13665,25 +13671,25 @@
         <v>101</v>
       </c>
       <c r="C418" s="1">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="D418" t="s">
-        <v>11</v>
+        <v>307</v>
       </c>
       <c r="E418" t="s">
-        <v>12</v>
+        <v>208</v>
       </c>
       <c r="F418">
-        <v>69343</v>
+        <v>69436</v>
       </c>
       <c r="G418">
-        <v>179180</v>
+        <v>179014</v>
       </c>
       <c r="H418" s="2">
-        <v>1281.22</v>
+        <v>804.72</v>
       </c>
       <c r="I418" s="1">
-        <v>46311</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="419" spans="1:9" x14ac:dyDescent="0.25">
@@ -13694,25 +13700,25 @@
         <v>101</v>
       </c>
       <c r="C419" s="1">
-        <v>46307</v>
+        <v>46304</v>
       </c>
       <c r="D419" t="s">
-        <v>297</v>
+        <v>308</v>
       </c>
       <c r="E419" t="s">
-        <v>298</v>
+        <v>309</v>
       </c>
       <c r="F419">
-        <v>69282</v>
+        <v>68124</v>
       </c>
       <c r="G419">
-        <v>179240</v>
+        <v>179016</v>
       </c>
       <c r="H419" s="2">
-        <v>6749.72</v>
+        <v>5155</v>
       </c>
       <c r="I419" s="1">
-        <v>46317</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="420" spans="1:9" x14ac:dyDescent="0.25">
@@ -13726,195 +13732,201 @@
         <v>46306</v>
       </c>
       <c r="D420" t="s">
-        <v>299</v>
+        <v>310</v>
       </c>
       <c r="E420" t="s">
         <v>43</v>
       </c>
       <c r="F420">
-        <v>67806</v>
+        <v>68499</v>
       </c>
       <c r="G420">
-        <v>179157</v>
+        <v>179177</v>
       </c>
       <c r="H420" s="2">
-        <v>2556</v>
+        <v>3763</v>
       </c>
       <c r="I420" s="1">
-        <v>46300</v>
+        <v>1</v>
       </c>
     </row>
     <row r="421" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A421" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B421">
         <v>101</v>
       </c>
       <c r="C421" s="1">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="D421" t="s">
-        <v>300</v>
+        <v>310</v>
       </c>
       <c r="E421" t="s">
-        <v>301</v>
+        <v>43</v>
       </c>
       <c r="F421">
-        <v>69774</v>
+        <v>69315</v>
       </c>
       <c r="G421">
-        <v>179269</v>
+        <v>179171</v>
       </c>
       <c r="H421" s="2">
-        <v>833.92</v>
+        <v>417.6</v>
       </c>
       <c r="I421" s="1">
-        <v>46308</v>
+        <v>46300</v>
       </c>
     </row>
     <row r="422" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A422" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B422">
         <v>101</v>
       </c>
       <c r="C422" s="1">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="D422" t="s">
-        <v>231</v>
+        <v>311</v>
       </c>
       <c r="E422" t="s">
-        <v>232</v>
+        <v>312</v>
+      </c>
+      <c r="F422">
+        <v>68459</v>
       </c>
       <c r="G422">
-        <v>179291</v>
+        <v>179159</v>
       </c>
       <c r="H422" s="2">
-        <v>1193.1099999999999</v>
+        <v>761.75</v>
+      </c>
+      <c r="I422" s="1">
+        <v>46287</v>
       </c>
     </row>
     <row r="423" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A423" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B423">
         <v>101</v>
       </c>
       <c r="C423" s="1">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="D423" t="s">
-        <v>416</v>
+        <v>19</v>
       </c>
       <c r="E423" t="s">
-        <v>417</v>
+        <v>20</v>
       </c>
       <c r="F423">
-        <v>68800</v>
+        <v>69517</v>
       </c>
       <c r="G423">
-        <v>179271</v>
+        <v>179165</v>
       </c>
       <c r="H423" s="2">
-        <v>1414.25</v>
+        <v>13.2</v>
       </c>
       <c r="I423" s="1">
-        <v>46293</v>
+        <v>46301</v>
       </c>
     </row>
     <row r="424" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A424" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B424">
         <v>101</v>
       </c>
       <c r="C424" s="1">
-        <v>46308</v>
+        <v>46306</v>
       </c>
       <c r="D424" t="s">
-        <v>54</v>
+        <v>313</v>
       </c>
       <c r="E424" t="s">
-        <v>55</v>
+        <v>314</v>
       </c>
       <c r="F424">
-        <v>69781</v>
+        <v>66362</v>
       </c>
       <c r="G424">
-        <v>179275</v>
+        <v>179186</v>
       </c>
       <c r="H424" s="2">
-        <v>1074</v>
+        <v>440</v>
       </c>
       <c r="I424" s="1">
-        <v>46308</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="425" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A425" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B425">
         <v>101</v>
       </c>
       <c r="C425" s="1">
-        <v>46303</v>
+        <v>46306</v>
       </c>
       <c r="D425" t="s">
-        <v>302</v>
+        <v>315</v>
       </c>
       <c r="E425" t="s">
-        <v>303</v>
+        <v>316</v>
       </c>
       <c r="F425">
-        <v>68896</v>
+        <v>66876</v>
       </c>
       <c r="G425">
-        <v>178889</v>
+        <v>179182</v>
       </c>
       <c r="H425" s="2">
-        <v>2700</v>
+        <v>2822.1</v>
       </c>
       <c r="I425" s="1">
-        <v>46294</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="426" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A426" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B426">
         <v>101</v>
       </c>
       <c r="C426" s="1">
-        <v>46303</v>
+        <v>46306</v>
       </c>
       <c r="D426" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="E426" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="F426">
-        <v>68897</v>
+        <v>69258</v>
       </c>
       <c r="G426">
-        <v>178938</v>
+        <v>179161</v>
       </c>
       <c r="H426" s="2">
-        <v>2700</v>
+        <v>128.69999999999999</v>
       </c>
       <c r="I426" s="1">
-        <v>46294</v>
+        <v>46297</v>
       </c>
     </row>
     <row r="427" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A427" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B427">
         <v>101</v>
@@ -13923,114 +13935,114 @@
         <v>46307</v>
       </c>
       <c r="D427" t="s">
-        <v>5</v>
+        <v>319</v>
       </c>
       <c r="E427" t="s">
-        <v>6</v>
+        <v>320</v>
       </c>
       <c r="F427">
-        <v>69193</v>
+        <v>69318</v>
       </c>
       <c r="G427">
-        <v>179202</v>
+        <v>179210</v>
       </c>
       <c r="H427" s="2">
-        <v>891</v>
+        <v>1126.24</v>
       </c>
       <c r="I427" s="1">
-        <v>46308</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="428" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A428" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B428">
         <v>101</v>
       </c>
       <c r="C428" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="D428" t="s">
-        <v>5</v>
+        <v>310</v>
       </c>
       <c r="E428" t="s">
-        <v>6</v>
+        <v>43</v>
       </c>
       <c r="F428">
-        <v>69291</v>
+        <v>68477</v>
       </c>
       <c r="G428">
-        <v>179203</v>
+        <v>179360</v>
       </c>
       <c r="H428" s="2">
-        <v>990</v>
+        <v>40740</v>
       </c>
       <c r="I428" s="1">
-        <v>46308</v>
+        <v>46287</v>
       </c>
     </row>
     <row r="429" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A429" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B429">
         <v>101</v>
       </c>
       <c r="C429" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="D429" t="s">
-        <v>134</v>
+        <v>321</v>
       </c>
       <c r="E429" t="s">
-        <v>135</v>
+        <v>322</v>
       </c>
       <c r="F429">
-        <v>69539</v>
+        <v>67697</v>
       </c>
       <c r="G429">
-        <v>178991</v>
+        <v>179278</v>
       </c>
       <c r="H429" s="2">
-        <v>161.04</v>
+        <v>1965.6</v>
       </c>
       <c r="I429" s="1">
-        <v>46303</v>
+        <v>46279</v>
       </c>
     </row>
     <row r="430" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A430" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B430">
         <v>101</v>
       </c>
       <c r="C430" s="1">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="D430" t="s">
-        <v>304</v>
+        <v>315</v>
       </c>
       <c r="E430" t="s">
-        <v>305</v>
+        <v>316</v>
       </c>
       <c r="F430">
-        <v>69782</v>
+        <v>69468</v>
       </c>
       <c r="G430">
-        <v>179212</v>
+        <v>179340</v>
       </c>
       <c r="H430" s="2">
-        <v>1164.4000000000001</v>
+        <v>1531.16</v>
       </c>
       <c r="I430" s="1">
-        <v>46304</v>
+        <v>46311</v>
       </c>
     </row>
     <row r="431" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A431" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B431">
         <v>101</v>
@@ -14039,16 +14051,22 @@
         <v>46308</v>
       </c>
       <c r="D431" t="s">
-        <v>123</v>
+        <v>323</v>
       </c>
       <c r="E431" t="s">
-        <v>124</v>
+        <v>324</v>
+      </c>
+      <c r="F431">
+        <v>69587</v>
       </c>
       <c r="G431">
-        <v>179286</v>
+        <v>179285</v>
       </c>
       <c r="H431" s="2">
-        <v>5236.78</v>
+        <v>1165.2</v>
+      </c>
+      <c r="I431" s="1">
+        <v>46304</v>
       </c>
     </row>
     <row r="432" spans="1:9" x14ac:dyDescent="0.25">
@@ -14062,22 +14080,16 @@
         <v>46308</v>
       </c>
       <c r="D432" t="s">
-        <v>306</v>
+        <v>44</v>
       </c>
       <c r="E432" t="s">
-        <v>99</v>
-      </c>
-      <c r="F432">
-        <v>69477</v>
+        <v>45</v>
       </c>
       <c r="G432">
-        <v>179273</v>
+        <v>179295</v>
       </c>
       <c r="H432" s="2">
-        <v>7943.55</v>
-      </c>
-      <c r="I432" s="1">
-        <v>46307</v>
+        <v>15485.79</v>
       </c>
     </row>
     <row r="433" spans="1:9" x14ac:dyDescent="0.25">
@@ -14091,22 +14103,22 @@
         <v>46308</v>
       </c>
       <c r="D433" t="s">
-        <v>130</v>
+        <v>44</v>
       </c>
       <c r="E433" t="s">
-        <v>131</v>
+        <v>45</v>
       </c>
       <c r="F433">
-        <v>69691</v>
+        <v>69945</v>
       </c>
       <c r="G433">
-        <v>179365</v>
+        <v>179294</v>
       </c>
       <c r="H433" s="2">
-        <v>248.9</v>
+        <v>2100</v>
       </c>
       <c r="I433" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="434" spans="1:9" x14ac:dyDescent="0.25">
@@ -14120,288 +14132,282 @@
         <v>46308</v>
       </c>
       <c r="D434" t="s">
-        <v>134</v>
+        <v>290</v>
       </c>
       <c r="E434" t="s">
-        <v>135</v>
+        <v>291</v>
       </c>
       <c r="F434">
-        <v>68186</v>
+        <v>69656</v>
       </c>
       <c r="G434">
-        <v>179268</v>
+        <v>179270</v>
       </c>
       <c r="H434" s="2">
-        <v>5692.68</v>
+        <v>283.60000000000002</v>
       </c>
       <c r="I434" s="1">
-        <v>46296</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="435" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A435" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B435">
         <v>101</v>
       </c>
       <c r="C435" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="D435" t="s">
-        <v>307</v>
+        <v>300</v>
       </c>
       <c r="E435" t="s">
-        <v>208</v>
+        <v>301</v>
       </c>
       <c r="F435">
-        <v>69436</v>
+        <v>69774</v>
       </c>
       <c r="G435">
-        <v>179014</v>
+        <v>179269</v>
       </c>
       <c r="H435" s="2">
-        <v>804.72</v>
+        <v>833.92</v>
       </c>
       <c r="I435" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="436" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A436" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B436">
         <v>101</v>
       </c>
       <c r="C436" s="1">
-        <v>46304</v>
+        <v>46308</v>
       </c>
       <c r="D436" t="s">
-        <v>308</v>
+        <v>231</v>
       </c>
       <c r="E436" t="s">
-        <v>309</v>
-      </c>
-      <c r="F436">
-        <v>68124</v>
+        <v>232</v>
       </c>
       <c r="G436">
-        <v>179016</v>
+        <v>179291</v>
       </c>
       <c r="H436" s="2">
-        <v>5155</v>
-      </c>
-      <c r="I436" s="1">
-        <v>46281</v>
+        <v>1193.1099999999999</v>
       </c>
     </row>
     <row r="437" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A437" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B437">
         <v>101</v>
       </c>
       <c r="C437" s="1">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="D437" t="s">
-        <v>310</v>
+        <v>416</v>
       </c>
       <c r="E437" t="s">
-        <v>43</v>
+        <v>417</v>
       </c>
       <c r="F437">
-        <v>68499</v>
+        <v>68800</v>
       </c>
       <c r="G437">
-        <v>179177</v>
+        <v>179271</v>
       </c>
       <c r="H437" s="2">
-        <v>3763</v>
+        <v>1414.25</v>
       </c>
       <c r="I437" s="1">
-        <v>1</v>
+        <v>46293</v>
       </c>
     </row>
     <row r="438" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A438" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B438">
         <v>101</v>
       </c>
       <c r="C438" s="1">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="D438" t="s">
-        <v>310</v>
+        <v>54</v>
       </c>
       <c r="E438" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="F438">
-        <v>69315</v>
+        <v>69781</v>
       </c>
       <c r="G438">
-        <v>179171</v>
+        <v>179275</v>
       </c>
       <c r="H438" s="2">
-        <v>417.6</v>
+        <v>1074</v>
       </c>
       <c r="I438" s="1">
-        <v>46300</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="439" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A439" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B439">
         <v>101</v>
       </c>
       <c r="C439" s="1">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="D439" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="E439" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
       <c r="F439">
-        <v>68459</v>
+        <v>68896</v>
       </c>
       <c r="G439">
-        <v>179159</v>
+        <v>178889</v>
       </c>
       <c r="H439" s="2">
-        <v>761.75</v>
+        <v>2700</v>
       </c>
       <c r="I439" s="1">
-        <v>46287</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="440" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A440" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B440">
         <v>101</v>
       </c>
       <c r="C440" s="1">
-        <v>46306</v>
+        <v>46303</v>
       </c>
       <c r="D440" t="s">
-        <v>19</v>
+        <v>302</v>
       </c>
       <c r="E440" t="s">
-        <v>20</v>
+        <v>303</v>
       </c>
       <c r="F440">
-        <v>69517</v>
+        <v>68897</v>
       </c>
       <c r="G440">
-        <v>179165</v>
+        <v>178938</v>
       </c>
       <c r="H440" s="2">
-        <v>13.2</v>
+        <v>2700</v>
       </c>
       <c r="I440" s="1">
-        <v>46301</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="441" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A441" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B441">
         <v>101</v>
       </c>
       <c r="C441" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="D441" t="s">
-        <v>313</v>
+        <v>5</v>
       </c>
       <c r="E441" t="s">
-        <v>314</v>
+        <v>6</v>
       </c>
       <c r="F441">
-        <v>66362</v>
+        <v>69193</v>
       </c>
       <c r="G441">
-        <v>179186</v>
+        <v>179202</v>
       </c>
       <c r="H441" s="2">
-        <v>440</v>
+        <v>891</v>
       </c>
       <c r="I441" s="1">
-        <v>46295</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="442" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A442" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B442">
         <v>101</v>
       </c>
       <c r="C442" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="D442" t="s">
-        <v>315</v>
+        <v>5</v>
       </c>
       <c r="E442" t="s">
-        <v>316</v>
+        <v>6</v>
       </c>
       <c r="F442">
-        <v>66876</v>
+        <v>69291</v>
       </c>
       <c r="G442">
-        <v>179182</v>
+        <v>179203</v>
       </c>
       <c r="H442" s="2">
-        <v>2822.1</v>
+        <v>990</v>
       </c>
       <c r="I442" s="1">
-        <v>46295</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="443" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A443" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B443">
         <v>101</v>
       </c>
       <c r="C443" s="1">
-        <v>46306</v>
+        <v>46304</v>
       </c>
       <c r="D443" t="s">
-        <v>317</v>
+        <v>134</v>
       </c>
       <c r="E443" t="s">
-        <v>318</v>
+        <v>135</v>
       </c>
       <c r="F443">
-        <v>69258</v>
+        <v>69539</v>
       </c>
       <c r="G443">
-        <v>179161</v>
+        <v>178991</v>
       </c>
       <c r="H443" s="2">
-        <v>128.69999999999999</v>
+        <v>161.04</v>
       </c>
       <c r="I443" s="1">
-        <v>46297</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="444" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A444" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B444">
         <v>101</v>
@@ -14410,27 +14416,27 @@
         <v>46307</v>
       </c>
       <c r="D444" t="s">
-        <v>319</v>
+        <v>304</v>
       </c>
       <c r="E444" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="F444">
-        <v>69318</v>
+        <v>69782</v>
       </c>
       <c r="G444">
-        <v>179210</v>
+        <v>179212</v>
       </c>
       <c r="H444" s="2">
-        <v>1126.24</v>
+        <v>1164.4000000000001</v>
       </c>
       <c r="I444" s="1">
-        <v>46303</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="445" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A445" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B445">
         <v>101</v>
@@ -14439,27 +14445,21 @@
         <v>46308</v>
       </c>
       <c r="D445" t="s">
-        <v>310</v>
+        <v>123</v>
       </c>
       <c r="E445" t="s">
-        <v>43</v>
-      </c>
-      <c r="F445">
-        <v>68477</v>
+        <v>124</v>
       </c>
       <c r="G445">
-        <v>179360</v>
+        <v>179286</v>
       </c>
       <c r="H445" s="2">
-        <v>40740</v>
-      </c>
-      <c r="I445" s="1">
-        <v>46287</v>
+        <v>5236.78</v>
       </c>
     </row>
     <row r="446" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A446" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B446">
         <v>101</v>
@@ -14468,27 +14468,27 @@
         <v>46308</v>
       </c>
       <c r="D446" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
       <c r="E446" t="s">
-        <v>322</v>
+        <v>99</v>
       </c>
       <c r="F446">
-        <v>67697</v>
+        <v>69477</v>
       </c>
       <c r="G446">
-        <v>179278</v>
+        <v>179273</v>
       </c>
       <c r="H446" s="2">
-        <v>1965.6</v>
+        <v>7943.55</v>
       </c>
       <c r="I446" s="1">
-        <v>46279</v>
+        <v>46307</v>
       </c>
     </row>
     <row r="447" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A447" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B447">
         <v>101</v>
@@ -14497,27 +14497,27 @@
         <v>46308</v>
       </c>
       <c r="D447" t="s">
-        <v>315</v>
+        <v>130</v>
       </c>
       <c r="E447" t="s">
-        <v>316</v>
+        <v>131</v>
       </c>
       <c r="F447">
-        <v>69468</v>
+        <v>69691</v>
       </c>
       <c r="G447">
-        <v>179340</v>
+        <v>179365</v>
       </c>
       <c r="H447" s="2">
-        <v>1531.16</v>
+        <v>248.9</v>
       </c>
       <c r="I447" s="1">
-        <v>46311</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="448" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A448" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B448">
         <v>101</v>
@@ -14526,22 +14526,22 @@
         <v>46308</v>
       </c>
       <c r="D448" t="s">
-        <v>323</v>
+        <v>134</v>
       </c>
       <c r="E448" t="s">
-        <v>324</v>
+        <v>135</v>
       </c>
       <c r="F448">
-        <v>69587</v>
+        <v>68186</v>
       </c>
       <c r="G448">
-        <v>179285</v>
+        <v>179268</v>
       </c>
       <c r="H448" s="2">
-        <v>1165.2</v>
+        <v>5692.68</v>
       </c>
       <c r="I448" s="1">
-        <v>46304</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="449" spans="1:9" x14ac:dyDescent="0.25">
@@ -17526,94 +17526,94 @@
     </row>
     <row r="553" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A553" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B553">
         <v>101</v>
       </c>
       <c r="C553" s="1">
-        <v>46301</v>
+        <v>46300</v>
       </c>
       <c r="D553" t="s">
-        <v>34</v>
+        <v>360</v>
       </c>
       <c r="E553" t="s">
-        <v>35</v>
+        <v>361</v>
       </c>
       <c r="F553">
-        <v>68369</v>
+        <v>67222</v>
       </c>
       <c r="G553">
-        <v>178768</v>
+        <v>178649</v>
       </c>
       <c r="H553" s="2">
-        <v>11873.92</v>
+        <v>3427.56</v>
       </c>
       <c r="I553" s="1">
-        <v>46289</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="554" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A554" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B554">
         <v>101</v>
       </c>
       <c r="C554" s="1">
-        <v>46302</v>
+        <v>46300</v>
       </c>
       <c r="D554" t="s">
-        <v>337</v>
+        <v>280</v>
       </c>
       <c r="E554" t="s">
-        <v>338</v>
+        <v>281</v>
       </c>
       <c r="F554">
-        <v>69787</v>
+        <v>67280</v>
       </c>
       <c r="G554">
-        <v>178860</v>
+        <v>178693</v>
       </c>
       <c r="H554" s="2">
-        <v>4200</v>
+        <v>1228.6199999999999</v>
       </c>
       <c r="I554" s="1">
-        <v>46303</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="555" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A555" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B555">
         <v>101</v>
       </c>
       <c r="C555" s="1">
-        <v>46303</v>
+        <v>46301</v>
       </c>
       <c r="D555" t="s">
-        <v>339</v>
+        <v>19</v>
       </c>
       <c r="E555" t="s">
-        <v>340</v>
+        <v>20</v>
       </c>
       <c r="F555">
-        <v>68666</v>
+        <v>69083</v>
       </c>
       <c r="G555">
-        <v>178879</v>
+        <v>178756</v>
       </c>
       <c r="H555" s="2">
-        <v>2016</v>
+        <v>1347.21</v>
       </c>
       <c r="I555" s="1">
-        <v>1</v>
+        <v>46294</v>
       </c>
     </row>
     <row r="556" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A556" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B556">
         <v>101</v>
@@ -17622,339 +17622,375 @@
         <v>46306</v>
       </c>
       <c r="D556" t="s">
-        <v>341</v>
+        <v>310</v>
       </c>
       <c r="E556" t="s">
-        <v>342</v>
+        <v>43</v>
       </c>
       <c r="F556">
-        <v>68724</v>
+        <v>69209</v>
       </c>
       <c r="G556">
-        <v>179158</v>
+        <v>179190</v>
       </c>
       <c r="H556" s="2">
-        <v>355</v>
+        <v>144</v>
       </c>
       <c r="I556" s="1">
-        <v>46300</v>
+        <v>46295</v>
       </c>
     </row>
     <row r="557" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A557" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B557">
         <v>101</v>
       </c>
       <c r="C557" s="1">
-        <v>46306</v>
+        <v>46307</v>
       </c>
       <c r="D557" t="s">
-        <v>343</v>
+        <v>362</v>
       </c>
       <c r="E557" t="s">
-        <v>344</v>
+        <v>363</v>
       </c>
       <c r="F557">
-        <v>68287</v>
+        <v>69557</v>
       </c>
       <c r="G557">
-        <v>179160</v>
+        <v>179258</v>
       </c>
       <c r="H557" s="2">
-        <v>237.2</v>
+        <v>2750.5</v>
       </c>
       <c r="I557" s="1">
-        <v>1</v>
+        <v>46304</v>
       </c>
     </row>
     <row r="558" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A558" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B558">
         <v>101</v>
       </c>
       <c r="C558" s="1">
-        <v>46308</v>
+        <v>46307</v>
       </c>
       <c r="D558" t="s">
-        <v>345</v>
+        <v>364</v>
       </c>
       <c r="E558" t="s">
-        <v>346</v>
+        <v>32</v>
       </c>
       <c r="F558">
-        <v>69001</v>
+        <v>69221</v>
       </c>
       <c r="G558">
-        <v>179364</v>
+        <v>179257</v>
       </c>
       <c r="H558" s="2">
-        <v>578.1</v>
+        <v>1377.66</v>
       </c>
       <c r="I558" s="1">
-        <v>46309</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="559" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A559" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B559">
         <v>101</v>
       </c>
       <c r="C559" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D559" t="s">
-        <v>34</v>
+        <v>365</v>
       </c>
       <c r="E559" t="s">
-        <v>35</v>
+        <v>32</v>
+      </c>
+      <c r="F559">
+        <v>69565</v>
       </c>
       <c r="G559">
-        <v>179393</v>
+        <v>179254</v>
       </c>
       <c r="H559" s="2">
-        <v>3131.08</v>
+        <v>1615.1</v>
+      </c>
+      <c r="I559" s="1">
+        <v>46304</v>
       </c>
     </row>
     <row r="560" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A560" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B560">
         <v>101</v>
       </c>
       <c r="C560" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D560" t="s">
-        <v>27</v>
+        <v>366</v>
       </c>
       <c r="E560" t="s">
-        <v>28</v>
+        <v>32</v>
+      </c>
+      <c r="F560">
+        <v>69568</v>
       </c>
       <c r="G560">
-        <v>179392</v>
+        <v>179256</v>
       </c>
       <c r="H560" s="2">
-        <v>4357.7700000000004</v>
+        <v>596.09</v>
+      </c>
+      <c r="I560" s="1">
+        <v>46304</v>
       </c>
     </row>
     <row r="561" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A561" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B561">
         <v>101</v>
       </c>
       <c r="C561" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D561" t="s">
-        <v>27</v>
+        <v>367</v>
       </c>
       <c r="E561" t="s">
-        <v>28</v>
+        <v>32</v>
+      </c>
+      <c r="F561">
+        <v>69675</v>
       </c>
       <c r="G561">
-        <v>179456</v>
+        <v>179253</v>
       </c>
       <c r="H561" s="2">
-        <v>35065.599999999999</v>
+        <v>646.72</v>
+      </c>
+      <c r="I561" s="1">
+        <v>46308</v>
       </c>
     </row>
     <row r="562" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A562" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B562">
         <v>101</v>
       </c>
       <c r="C562" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D562" t="s">
-        <v>27</v>
+        <v>368</v>
       </c>
       <c r="E562" t="s">
-        <v>28</v>
+        <v>369</v>
       </c>
       <c r="F562">
-        <v>68993</v>
+        <v>69644</v>
       </c>
       <c r="G562">
-        <v>179398</v>
+        <v>179246</v>
       </c>
       <c r="H562" s="2">
-        <v>141.94</v>
+        <v>667.2</v>
       </c>
       <c r="I562" s="1">
-        <v>46303</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="563" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A563" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B563">
         <v>101</v>
       </c>
       <c r="C563" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D563" t="s">
-        <v>31</v>
+        <v>370</v>
       </c>
       <c r="E563" t="s">
-        <v>32</v>
+        <v>184</v>
+      </c>
+      <c r="F563">
+        <v>69558</v>
       </c>
       <c r="G563">
-        <v>179373</v>
+        <v>179255</v>
       </c>
       <c r="H563" s="2">
-        <v>1219.98</v>
+        <v>568.62</v>
+      </c>
+      <c r="I563" s="1">
+        <v>46304</v>
       </c>
     </row>
     <row r="564" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A564" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B564">
         <v>101</v>
       </c>
       <c r="C564" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D564" t="s">
-        <v>33</v>
+        <v>311</v>
       </c>
       <c r="E564" t="s">
-        <v>32</v>
+        <v>312</v>
       </c>
       <c r="F564">
-        <v>69275</v>
+        <v>68453</v>
       </c>
       <c r="G564">
-        <v>179399</v>
+        <v>179247</v>
       </c>
       <c r="H564" s="2">
-        <v>762.9</v>
+        <v>3241.96</v>
       </c>
       <c r="I564" s="1">
-        <v>46296</v>
+        <v>46286</v>
       </c>
     </row>
     <row r="565" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A565" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B565">
         <v>101</v>
       </c>
       <c r="C565" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D565" t="s">
-        <v>347</v>
+        <v>311</v>
       </c>
       <c r="E565" t="s">
-        <v>32</v>
+        <v>312</v>
+      </c>
+      <c r="F565">
+        <v>68454</v>
       </c>
       <c r="G565">
-        <v>179394</v>
+        <v>179248</v>
       </c>
       <c r="H565" s="2">
-        <v>1647.31</v>
+        <v>2480.21</v>
+      </c>
+      <c r="I565" s="1">
+        <v>46286</v>
       </c>
     </row>
     <row r="566" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A566" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B566">
         <v>101</v>
       </c>
       <c r="C566" s="1">
-        <v>46309</v>
+        <v>46307</v>
       </c>
       <c r="D566" t="s">
-        <v>341</v>
+        <v>371</v>
       </c>
       <c r="E566" t="s">
-        <v>342</v>
+        <v>372</v>
+      </c>
+      <c r="F566">
+        <v>67396</v>
       </c>
       <c r="G566">
-        <v>179377</v>
+        <v>179249</v>
       </c>
       <c r="H566" s="2">
-        <v>4762.8</v>
+        <v>1991.6</v>
+      </c>
+      <c r="I566" s="1">
+        <v>46287</v>
       </c>
     </row>
     <row r="567" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A567" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B567">
         <v>101</v>
       </c>
       <c r="C567" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="D567" t="s">
-        <v>341</v>
+        <v>310</v>
       </c>
       <c r="E567" t="s">
-        <v>342</v>
+        <v>43</v>
       </c>
       <c r="F567">
-        <v>68902</v>
+        <v>69713</v>
       </c>
       <c r="G567">
-        <v>179414</v>
+        <v>179315</v>
       </c>
       <c r="H567" s="2">
-        <v>200</v>
+        <v>6683.04</v>
       </c>
       <c r="I567" s="1">
-        <v>46296</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="568" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A568" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B568">
         <v>101</v>
       </c>
       <c r="C568" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="D568" t="s">
-        <v>341</v>
+        <v>310</v>
       </c>
       <c r="E568" t="s">
-        <v>342</v>
+        <v>43</v>
       </c>
       <c r="F568">
-        <v>69316</v>
+        <v>69923</v>
       </c>
       <c r="G568">
-        <v>179375</v>
+        <v>179280</v>
       </c>
       <c r="H568" s="2">
-        <v>453.6</v>
+        <v>5800</v>
       </c>
       <c r="I568" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
     </row>
     <row r="569" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A569" s="1">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B569">
         <v>101</v>
@@ -17963,51 +17999,45 @@
         <v>46309</v>
       </c>
       <c r="D569" t="s">
-        <v>341</v>
+        <v>373</v>
       </c>
       <c r="E569" t="s">
-        <v>342</v>
-      </c>
-      <c r="F569">
-        <v>69498</v>
+        <v>374</v>
       </c>
       <c r="G569">
-        <v>179371</v>
+        <v>179397</v>
       </c>
       <c r="H569" s="2">
-        <v>850.4</v>
-      </c>
-      <c r="I569" s="1">
-        <v>46309</v>
+        <v>1668.01</v>
       </c>
     </row>
     <row r="570" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A570" s="1">
+        <v>46309</v>
+      </c>
+      <c r="B570">
+        <v>101</v>
+      </c>
+      <c r="C570" s="1">
+        <v>46309</v>
+      </c>
+      <c r="D570" t="s">
+        <v>375</v>
+      </c>
+      <c r="E570" t="s">
+        <v>376</v>
+      </c>
+      <c r="F570">
+        <v>69894</v>
+      </c>
+      <c r="G570">
+        <v>179395</v>
+      </c>
+      <c r="H570" s="2">
+        <v>3165</v>
+      </c>
+      <c r="I570" s="1">
         <v>46310</v>
-      </c>
-      <c r="B570">
-        <v>101</v>
-      </c>
-      <c r="C570" s="1">
-        <v>46309</v>
-      </c>
-      <c r="D570" t="s">
-        <v>341</v>
-      </c>
-      <c r="E570" t="s">
-        <v>342</v>
-      </c>
-      <c r="F570">
-        <v>69795</v>
-      </c>
-      <c r="G570">
-        <v>179389</v>
-      </c>
-      <c r="H570" s="2">
-        <v>284</v>
-      </c>
-      <c r="I570" s="1">
-        <v>46309</v>
       </c>
     </row>
     <row r="571" spans="1:9" x14ac:dyDescent="0.25">
@@ -18018,25 +18048,25 @@
         <v>101</v>
       </c>
       <c r="C571" s="1">
-        <v>46309</v>
+        <v>46301</v>
       </c>
       <c r="D571" t="s">
-        <v>341</v>
+        <v>34</v>
       </c>
       <c r="E571" t="s">
-        <v>342</v>
+        <v>35</v>
       </c>
       <c r="F571">
-        <v>69842</v>
+        <v>68369</v>
       </c>
       <c r="G571">
-        <v>179388</v>
+        <v>178768</v>
       </c>
       <c r="H571" s="2">
-        <v>84</v>
+        <v>11873.92</v>
       </c>
       <c r="I571" s="1">
-        <v>46309</v>
+        <v>46289</v>
       </c>
     </row>
     <row r="572" spans="1:9" x14ac:dyDescent="0.25">
@@ -18047,25 +18077,25 @@
         <v>101</v>
       </c>
       <c r="C572" s="1">
-        <v>46309</v>
+        <v>46302</v>
       </c>
       <c r="D572" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
       <c r="E572" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="F572">
-        <v>69792</v>
+        <v>69787</v>
       </c>
       <c r="G572">
-        <v>179374</v>
+        <v>178860</v>
       </c>
       <c r="H572" s="2">
-        <v>4762.8</v>
+        <v>4200</v>
       </c>
       <c r="I572" s="1">
-        <v>46309</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="573" spans="1:9" x14ac:dyDescent="0.25">
@@ -18076,19 +18106,25 @@
         <v>101</v>
       </c>
       <c r="C573" s="1">
-        <v>46309</v>
+        <v>46303</v>
       </c>
       <c r="D573" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="E573" t="s">
-        <v>344</v>
+        <v>340</v>
+      </c>
+      <c r="F573">
+        <v>68666</v>
       </c>
       <c r="G573">
-        <v>179441</v>
+        <v>178879</v>
       </c>
       <c r="H573" s="2">
-        <v>1749.84</v>
+        <v>2016</v>
+      </c>
+      <c r="I573" s="1">
+        <v>1</v>
       </c>
     </row>
     <row r="574" spans="1:9" x14ac:dyDescent="0.25">
@@ -18099,19 +18135,25 @@
         <v>101</v>
       </c>
       <c r="C574" s="1">
-        <v>46309</v>
+        <v>46306</v>
       </c>
       <c r="D574" t="s">
-        <v>350</v>
+        <v>341</v>
       </c>
       <c r="E574" t="s">
-        <v>351</v>
+        <v>342</v>
+      </c>
+      <c r="F574">
+        <v>68724</v>
       </c>
       <c r="G574">
-        <v>179415</v>
+        <v>179158</v>
       </c>
       <c r="H574" s="2">
-        <v>4759.8999999999996</v>
+        <v>355</v>
+      </c>
+      <c r="I574" s="1">
+        <v>46300</v>
       </c>
     </row>
     <row r="575" spans="1:9" x14ac:dyDescent="0.25">
@@ -18122,25 +18164,25 @@
         <v>101</v>
       </c>
       <c r="C575" s="1">
-        <v>46309</v>
+        <v>46306</v>
       </c>
       <c r="D575" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="E575" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="F575">
-        <v>68807</v>
+        <v>68287</v>
       </c>
       <c r="G575">
-        <v>179413</v>
+        <v>179160</v>
       </c>
       <c r="H575" s="2">
-        <v>2147.5500000000002</v>
+        <v>237.2</v>
       </c>
       <c r="I575" s="1">
-        <v>46309</v>
+        <v>1</v>
       </c>
     </row>
     <row r="576" spans="1:9" x14ac:dyDescent="0.25">
@@ -18151,22 +18193,22 @@
         <v>101</v>
       </c>
       <c r="C576" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="D576" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="E576" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="F576">
-        <v>68809</v>
+        <v>69001</v>
       </c>
       <c r="G576">
-        <v>179391</v>
+        <v>179364</v>
       </c>
       <c r="H576" s="2">
-        <v>923</v>
+        <v>578.1</v>
       </c>
       <c r="I576" s="1">
         <v>46309</v>
@@ -18183,22 +18225,16 @@
         <v>46309</v>
       </c>
       <c r="D577" t="s">
-        <v>350</v>
+        <v>34</v>
       </c>
       <c r="E577" t="s">
-        <v>351</v>
-      </c>
-      <c r="F577">
-        <v>69370</v>
+        <v>35</v>
       </c>
       <c r="G577">
-        <v>179400</v>
+        <v>179393</v>
       </c>
       <c r="H577" s="2">
-        <v>1903.5</v>
-      </c>
-      <c r="I577" s="1">
-        <v>46309</v>
+        <v>3131.08</v>
       </c>
     </row>
     <row r="578" spans="1:9" x14ac:dyDescent="0.25">
@@ -18212,22 +18248,16 @@
         <v>46309</v>
       </c>
       <c r="D578" t="s">
-        <v>350</v>
+        <v>27</v>
       </c>
       <c r="E578" t="s">
-        <v>351</v>
-      </c>
-      <c r="F578">
-        <v>69778</v>
+        <v>28</v>
       </c>
       <c r="G578">
-        <v>179433</v>
+        <v>179392</v>
       </c>
       <c r="H578" s="2">
-        <v>600</v>
-      </c>
-      <c r="I578" s="1">
-        <v>46309</v>
+        <v>4357.7700000000004</v>
       </c>
     </row>
     <row r="579" spans="1:9" x14ac:dyDescent="0.25">
@@ -18235,28 +18265,22 @@
         <v>46310</v>
       </c>
       <c r="B579">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C579" s="1">
-        <v>45222</v>
+        <v>46309</v>
       </c>
       <c r="D579" t="s">
-        <v>352</v>
+        <v>27</v>
       </c>
       <c r="E579" t="s">
-        <v>353</v>
-      </c>
-      <c r="F579">
-        <v>450</v>
+        <v>28</v>
       </c>
       <c r="G579">
-        <v>514</v>
+        <v>179456</v>
       </c>
       <c r="H579" s="2">
-        <v>125.82</v>
-      </c>
-      <c r="I579" s="1">
-        <v>45222</v>
+        <v>35065.599999999999</v>
       </c>
     </row>
     <row r="580" spans="1:9" x14ac:dyDescent="0.25">
@@ -18264,28 +18288,28 @@
         <v>46310</v>
       </c>
       <c r="B580">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C580" s="1">
-        <v>45222</v>
+        <v>46309</v>
       </c>
       <c r="D580" t="s">
-        <v>354</v>
+        <v>27</v>
       </c>
       <c r="E580" t="s">
-        <v>208</v>
+        <v>28</v>
       </c>
       <c r="F580">
-        <v>459</v>
+        <v>68993</v>
       </c>
       <c r="G580">
-        <v>516</v>
+        <v>179398</v>
       </c>
       <c r="H580" s="2">
-        <v>898.2</v>
+        <v>141.94</v>
       </c>
       <c r="I580" s="1">
-        <v>45222</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="581" spans="1:9" x14ac:dyDescent="0.25">
@@ -18296,25 +18320,19 @@
         <v>101</v>
       </c>
       <c r="C581" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="D581" t="s">
-        <v>271</v>
+        <v>31</v>
       </c>
       <c r="E581" t="s">
-        <v>272</v>
-      </c>
-      <c r="F581">
-        <v>68599</v>
+        <v>32</v>
       </c>
       <c r="G581">
-        <v>179200</v>
+        <v>179373</v>
       </c>
       <c r="H581" s="2">
-        <v>2384.5700000000002</v>
-      </c>
-      <c r="I581" s="1">
-        <v>46296</v>
+        <v>1219.98</v>
       </c>
     </row>
     <row r="582" spans="1:9" x14ac:dyDescent="0.25">
@@ -18328,22 +18346,22 @@
         <v>46309</v>
       </c>
       <c r="D582" t="s">
-        <v>355</v>
+        <v>33</v>
       </c>
       <c r="E582" t="s">
         <v>32</v>
       </c>
       <c r="F582">
-        <v>69955</v>
+        <v>69275</v>
       </c>
       <c r="G582">
-        <v>179430</v>
+        <v>179399</v>
       </c>
       <c r="H582" s="2">
-        <v>1594.8</v>
+        <v>762.9</v>
       </c>
       <c r="I582" s="1">
-        <v>46310</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="583" spans="1:9" x14ac:dyDescent="0.25">
@@ -18357,22 +18375,16 @@
         <v>46309</v>
       </c>
       <c r="D583" t="s">
-        <v>356</v>
+        <v>347</v>
       </c>
       <c r="E583" t="s">
-        <v>357</v>
-      </c>
-      <c r="F583">
-        <v>69869</v>
+        <v>32</v>
       </c>
       <c r="G583">
-        <v>179384</v>
+        <v>179394</v>
       </c>
       <c r="H583" s="2">
-        <v>392.4</v>
-      </c>
-      <c r="I583" s="1">
-        <v>46309</v>
+        <v>1647.31</v>
       </c>
     </row>
     <row r="584" spans="1:9" x14ac:dyDescent="0.25">
@@ -18386,22 +18398,16 @@
         <v>46309</v>
       </c>
       <c r="D584" t="s">
-        <v>358</v>
+        <v>341</v>
       </c>
       <c r="E584" t="s">
-        <v>359</v>
-      </c>
-      <c r="F584">
-        <v>69663</v>
+        <v>342</v>
       </c>
       <c r="G584">
-        <v>179387</v>
+        <v>179377</v>
       </c>
       <c r="H584" s="2">
-        <v>1771.2</v>
-      </c>
-      <c r="I584" s="1">
-        <v>46309</v>
+        <v>4762.8</v>
       </c>
     </row>
     <row r="585" spans="1:9" x14ac:dyDescent="0.25">
@@ -18415,22 +18421,22 @@
         <v>46309</v>
       </c>
       <c r="D585" t="s">
-        <v>151</v>
+        <v>341</v>
       </c>
       <c r="E585" t="s">
-        <v>49</v>
+        <v>342</v>
       </c>
       <c r="F585">
-        <v>70060</v>
+        <v>68902</v>
       </c>
       <c r="G585">
-        <v>179435</v>
+        <v>179414</v>
       </c>
       <c r="H585" s="2">
-        <v>1406.66</v>
+        <v>200</v>
       </c>
       <c r="I585" s="1">
-        <v>46310</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="586" spans="1:9" x14ac:dyDescent="0.25">
@@ -18441,488 +18447,482 @@
         <v>101</v>
       </c>
       <c r="C586" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="D586" t="s">
-        <v>58</v>
+        <v>341</v>
       </c>
       <c r="E586" t="s">
-        <v>59</v>
+        <v>342</v>
+      </c>
+      <c r="F586">
+        <v>69316</v>
       </c>
       <c r="G586">
-        <v>179369</v>
+        <v>179375</v>
       </c>
       <c r="H586" s="2">
-        <v>26935.55</v>
+        <v>453.6</v>
+      </c>
+      <c r="I586" s="1">
+        <v>46309</v>
       </c>
     </row>
     <row r="587" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A587" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B587">
         <v>101</v>
       </c>
       <c r="C587" s="1">
-        <v>46300</v>
+        <v>46309</v>
       </c>
       <c r="D587" t="s">
-        <v>360</v>
+        <v>341</v>
       </c>
       <c r="E587" t="s">
-        <v>361</v>
+        <v>342</v>
       </c>
       <c r="F587">
-        <v>67222</v>
+        <v>69498</v>
       </c>
       <c r="G587">
-        <v>178649</v>
+        <v>179371</v>
       </c>
       <c r="H587" s="2">
-        <v>3427.56</v>
+        <v>850.4</v>
       </c>
       <c r="I587" s="1">
-        <v>46294</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="588" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A588" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B588">
         <v>101</v>
       </c>
       <c r="C588" s="1">
-        <v>46300</v>
+        <v>46309</v>
       </c>
       <c r="D588" t="s">
-        <v>280</v>
+        <v>341</v>
       </c>
       <c r="E588" t="s">
-        <v>281</v>
+        <v>342</v>
       </c>
       <c r="F588">
-        <v>67280</v>
+        <v>69795</v>
       </c>
       <c r="G588">
-        <v>178693</v>
+        <v>179389</v>
       </c>
       <c r="H588" s="2">
-        <v>1228.6199999999999</v>
+        <v>284</v>
       </c>
       <c r="I588" s="1">
-        <v>46294</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="589" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A589" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B589">
         <v>101</v>
       </c>
       <c r="C589" s="1">
-        <v>46301</v>
+        <v>46309</v>
       </c>
       <c r="D589" t="s">
-        <v>19</v>
+        <v>341</v>
       </c>
       <c r="E589" t="s">
-        <v>20</v>
+        <v>342</v>
       </c>
       <c r="F589">
-        <v>69083</v>
+        <v>69842</v>
       </c>
       <c r="G589">
-        <v>178756</v>
+        <v>179388</v>
       </c>
       <c r="H589" s="2">
-        <v>1347.21</v>
+        <v>84</v>
       </c>
       <c r="I589" s="1">
-        <v>46294</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="590" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A590" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B590">
         <v>101</v>
       </c>
       <c r="C590" s="1">
-        <v>46306</v>
+        <v>46309</v>
       </c>
       <c r="D590" t="s">
-        <v>310</v>
+        <v>348</v>
       </c>
       <c r="E590" t="s">
-        <v>43</v>
+        <v>349</v>
       </c>
       <c r="F590">
-        <v>69209</v>
+        <v>69792</v>
       </c>
       <c r="G590">
-        <v>179190</v>
+        <v>179374</v>
       </c>
       <c r="H590" s="2">
-        <v>144</v>
+        <v>4762.8</v>
       </c>
       <c r="I590" s="1">
-        <v>46295</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="591" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A591" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B591">
         <v>101</v>
       </c>
       <c r="C591" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D591" t="s">
-        <v>362</v>
+        <v>343</v>
       </c>
       <c r="E591" t="s">
-        <v>363</v>
-      </c>
-      <c r="F591">
-        <v>69557</v>
+        <v>344</v>
       </c>
       <c r="G591">
-        <v>179258</v>
+        <v>179441</v>
       </c>
       <c r="H591" s="2">
-        <v>2750.5</v>
-      </c>
-      <c r="I591" s="1">
-        <v>46304</v>
+        <v>1749.84</v>
       </c>
     </row>
     <row r="592" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A592" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B592">
         <v>101</v>
       </c>
       <c r="C592" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D592" t="s">
-        <v>364</v>
+        <v>350</v>
       </c>
       <c r="E592" t="s">
-        <v>32</v>
-      </c>
-      <c r="F592">
-        <v>69221</v>
+        <v>351</v>
       </c>
       <c r="G592">
-        <v>179257</v>
+        <v>179415</v>
       </c>
       <c r="H592" s="2">
-        <v>1377.66</v>
-      </c>
-      <c r="I592" s="1">
-        <v>46296</v>
+        <v>4759.8999999999996</v>
       </c>
     </row>
     <row r="593" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A593" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B593">
         <v>101</v>
       </c>
       <c r="C593" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D593" t="s">
-        <v>365</v>
+        <v>350</v>
       </c>
       <c r="E593" t="s">
-        <v>32</v>
+        <v>351</v>
       </c>
       <c r="F593">
-        <v>69565</v>
+        <v>68807</v>
       </c>
       <c r="G593">
-        <v>179254</v>
+        <v>179413</v>
       </c>
       <c r="H593" s="2">
-        <v>1615.1</v>
+        <v>2147.5500000000002</v>
       </c>
       <c r="I593" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="594" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A594" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B594">
         <v>101</v>
       </c>
       <c r="C594" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D594" t="s">
-        <v>366</v>
+        <v>350</v>
       </c>
       <c r="E594" t="s">
-        <v>32</v>
+        <v>351</v>
       </c>
       <c r="F594">
-        <v>69568</v>
+        <v>68809</v>
       </c>
       <c r="G594">
-        <v>179256</v>
+        <v>179391</v>
       </c>
       <c r="H594" s="2">
-        <v>596.09</v>
+        <v>923</v>
       </c>
       <c r="I594" s="1">
-        <v>46304</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="595" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A595" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B595">
         <v>101</v>
       </c>
       <c r="C595" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D595" t="s">
-        <v>367</v>
+        <v>350</v>
       </c>
       <c r="E595" t="s">
-        <v>32</v>
+        <v>351</v>
       </c>
       <c r="F595">
-        <v>69675</v>
+        <v>69370</v>
       </c>
       <c r="G595">
-        <v>179253</v>
+        <v>179400</v>
       </c>
       <c r="H595" s="2">
-        <v>646.72</v>
+        <v>1903.5</v>
       </c>
       <c r="I595" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="596" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A596" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B596">
         <v>101</v>
       </c>
       <c r="C596" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D596" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="E596" t="s">
-        <v>369</v>
+        <v>351</v>
       </c>
       <c r="F596">
-        <v>69644</v>
+        <v>69778</v>
       </c>
       <c r="G596">
-        <v>179246</v>
+        <v>179433</v>
       </c>
       <c r="H596" s="2">
-        <v>667.2</v>
+        <v>600</v>
       </c>
       <c r="I596" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="597" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A597" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B597">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C597" s="1">
-        <v>46307</v>
+        <v>45222</v>
       </c>
       <c r="D597" t="s">
-        <v>370</v>
+        <v>352</v>
       </c>
       <c r="E597" t="s">
-        <v>184</v>
+        <v>353</v>
       </c>
       <c r="F597">
-        <v>69558</v>
+        <v>450</v>
       </c>
       <c r="G597">
-        <v>179255</v>
+        <v>514</v>
       </c>
       <c r="H597" s="2">
-        <v>568.62</v>
+        <v>125.82</v>
       </c>
       <c r="I597" s="1">
-        <v>46304</v>
+        <v>45222</v>
       </c>
     </row>
     <row r="598" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A598" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B598">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C598" s="1">
-        <v>46307</v>
+        <v>45222</v>
       </c>
       <c r="D598" t="s">
-        <v>311</v>
+        <v>354</v>
       </c>
       <c r="E598" t="s">
-        <v>312</v>
+        <v>208</v>
       </c>
       <c r="F598">
-        <v>68453</v>
+        <v>459</v>
       </c>
       <c r="G598">
-        <v>179247</v>
+        <v>516</v>
       </c>
       <c r="H598" s="2">
-        <v>3241.96</v>
+        <v>898.2</v>
       </c>
       <c r="I598" s="1">
-        <v>46286</v>
+        <v>45222</v>
       </c>
     </row>
     <row r="599" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A599" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B599">
         <v>101</v>
       </c>
       <c r="C599" s="1">
-        <v>46307</v>
+        <v>46306</v>
       </c>
       <c r="D599" t="s">
-        <v>311</v>
+        <v>271</v>
       </c>
       <c r="E599" t="s">
-        <v>312</v>
+        <v>272</v>
       </c>
       <c r="F599">
-        <v>68454</v>
+        <v>68599</v>
       </c>
       <c r="G599">
-        <v>179248</v>
+        <v>179200</v>
       </c>
       <c r="H599" s="2">
-        <v>2480.21</v>
+        <v>2384.5700000000002</v>
       </c>
       <c r="I599" s="1">
-        <v>46286</v>
+        <v>46296</v>
       </c>
     </row>
     <row r="600" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A600" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B600">
         <v>101</v>
       </c>
       <c r="C600" s="1">
-        <v>46307</v>
+        <v>46309</v>
       </c>
       <c r="D600" t="s">
-        <v>371</v>
+        <v>355</v>
       </c>
       <c r="E600" t="s">
-        <v>372</v>
+        <v>32</v>
       </c>
       <c r="F600">
-        <v>67396</v>
+        <v>69955</v>
       </c>
       <c r="G600">
-        <v>179249</v>
+        <v>179430</v>
       </c>
       <c r="H600" s="2">
-        <v>1991.6</v>
+        <v>1594.8</v>
       </c>
       <c r="I600" s="1">
-        <v>46287</v>
+        <v>46310</v>
       </c>
     </row>
     <row r="601" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A601" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B601">
         <v>101</v>
       </c>
       <c r="C601" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="D601" t="s">
-        <v>310</v>
+        <v>356</v>
       </c>
       <c r="E601" t="s">
-        <v>43</v>
+        <v>357</v>
       </c>
       <c r="F601">
-        <v>69713</v>
+        <v>69869</v>
       </c>
       <c r="G601">
-        <v>179315</v>
+        <v>179384</v>
       </c>
       <c r="H601" s="2">
-        <v>6683.04</v>
+        <v>392.4</v>
       </c>
       <c r="I601" s="1">
-        <v>46303</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="602" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A602" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B602">
         <v>101</v>
       </c>
       <c r="C602" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="D602" t="s">
-        <v>310</v>
+        <v>358</v>
       </c>
       <c r="E602" t="s">
-        <v>43</v>
+        <v>359</v>
       </c>
       <c r="F602">
-        <v>69923</v>
+        <v>69663</v>
       </c>
       <c r="G602">
-        <v>179280</v>
+        <v>179387</v>
       </c>
       <c r="H602" s="2">
-        <v>5800</v>
+        <v>1771.2</v>
       </c>
       <c r="I602" s="1">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row r="603" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A603" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B603">
         <v>101</v>
@@ -18931,45 +18931,45 @@
         <v>46309</v>
       </c>
       <c r="D603" t="s">
-        <v>373</v>
+        <v>151</v>
       </c>
       <c r="E603" t="s">
-        <v>374</v>
+        <v>49</v>
+      </c>
+      <c r="F603">
+        <v>70060</v>
       </c>
       <c r="G603">
-        <v>179397</v>
+        <v>179435</v>
       </c>
       <c r="H603" s="2">
-        <v>1668.01</v>
+        <v>1406.66</v>
+      </c>
+      <c r="I603" s="1">
+        <v>46310</v>
       </c>
     </row>
     <row r="604" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A604" s="1">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B604">
         <v>101</v>
       </c>
       <c r="C604" s="1">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="D604" t="s">
-        <v>375</v>
+        <v>58</v>
       </c>
       <c r="E604" t="s">
-        <v>376</v>
-      </c>
-      <c r="F604">
-        <v>69894</v>
+        <v>59</v>
       </c>
       <c r="G604">
-        <v>179395</v>
+        <v>179369</v>
       </c>
       <c r="H604" s="2">
-        <v>3165</v>
-      </c>
-      <c r="I604" s="1">
-        <v>46310</v>
+        <v>26935.55</v>
       </c>
     </row>
     <row r="605" spans="1:9" x14ac:dyDescent="0.25">
@@ -22242,6 +22242,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:I719">
+    <sortCondition ref="A703:A719"/>
+  </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: Modificações para leitura nos dados e inclusão da biblioteca de Machine Learning
</commit_message>
<xml_diff>
--- a/DadosRomaneios.xlsx
+++ b/DadosRomaneios.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.andrade\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CE11EF9-5BEB-4AF9-B4B3-109DCC56BD26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B97880-BCEF-486C-9ADF-DBCD7F7C6AF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
+    <workbookView xWindow="16284" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Romaneios" sheetId="2" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,8 +39,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1445" uniqueCount="421">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1446" uniqueCount="422">
   <si>
     <t>000024 - 021</t>
   </si>
@@ -1302,6 +1325,9 @@
   </si>
   <si>
     <t>AFIP CLEMENTINO</t>
+  </si>
+  <si>
+    <t>Qtd. Expedição</t>
   </si>
 </sst>
 </file>
@@ -1311,13 +1337,19 @@
   <numFmts count="1">
     <numFmt numFmtId="8" formatCode="&quot;R$&quot;\ #,##0.00;[Red]\-&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1340,10 +1372,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22248,4 +22281,118 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5180BF9C-1943-4030-8A1B-6F86FE205C17}">
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="str" cm="1">
+        <f t="array" ref="A1:A11">_xlfn.UNIQUE(Romaneios!A1:A719)</f>
+        <v>Dt. Romaneio</v>
+      </c>
+      <c r="B1" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>46302</v>
+      </c>
+      <c r="B2">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A2)</f>
+        <v>35</v>
+      </c>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>46303</v>
+      </c>
+      <c r="B3">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A3)</f>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>46304</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A4)</f>
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>46305</v>
+      </c>
+      <c r="B5">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A5)</f>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>46306</v>
+      </c>
+      <c r="B6">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A6)</f>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>46307</v>
+      </c>
+      <c r="B7">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A7)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>46308</v>
+      </c>
+      <c r="B8">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A8)</f>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>46309</v>
+      </c>
+      <c r="B9">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A9)</f>
+        <v>139</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>46310</v>
+      </c>
+      <c r="B10">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A10)</f>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
+        <v>46311</v>
+      </c>
+      <c r="B11">
+        <f>COUNTIF(Romaneios!A:A,Planilha1!A11)</f>
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: Atualização de dados faltantes
</commit_message>
<xml_diff>
--- a/DadosRomaneios.xlsx
+++ b/DadosRomaneios.xlsx
@@ -8,18 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14689DD-72CB-4E34-B996-5F058AE252BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2022B6CC-C9D8-4A70-A37C-2BF50ED79ADB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
   </bookViews>
   <sheets>
     <sheet name="Romaneios" sheetId="2" r:id="rId1"/>
     <sheet name="DadosRomaneios" sheetId="3" r:id="rId2"/>
-    <sheet name="Planilha1" sheetId="4" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Planilha1!$A$1:$D$128</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -44,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="923" uniqueCount="208">
   <si>
     <t>ALBERT EINSTEIN</t>
   </si>
@@ -16462,7 +16458,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5180BF9C-1943-4030-8A1B-6F86FE205C17}">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -16471,7 +16467,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="str" cm="1">
-        <f t="array" ref="A1:A14">_xlfn.UNIQUE(Romaneios!A1:A791)</f>
+        <f t="array" ref="A1:A15">_xlfn.UNIQUE(Romaneios!A1:A918)</f>
         <v>Dt. Romaneio</v>
       </c>
       <c r="B1" t="s">
@@ -16596,1768 +16592,16 @@
         <v>69</v>
       </c>
     </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>46315</v>
+      </c>
+      <c r="B15">
+        <f>COUNTIF(Romaneios!A:A,DadosRomaneios!A15)</f>
+        <v>127</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCA1778-A08A-4BBC-894B-FE6DC9B4E104}">
-  <dimension ref="A1:D128"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="15.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>168</v>
-      </c>
-      <c r="B1" t="s">
-        <v>170</v>
-      </c>
-      <c r="C1" t="s">
-        <v>171</v>
-      </c>
-      <c r="D1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2">
-        <v>70278</v>
-      </c>
-      <c r="D2">
-        <v>179693</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>179705</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C4">
-        <v>70279</v>
-      </c>
-      <c r="D4">
-        <v>179692</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B5" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>70298</v>
-      </c>
-      <c r="D5">
-        <v>179680</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B6" t="s">
-        <v>94</v>
-      </c>
-      <c r="D6">
-        <v>179646</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B7" t="s">
-        <v>190</v>
-      </c>
-      <c r="C7">
-        <v>70059</v>
-      </c>
-      <c r="D7">
-        <v>179565</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8">
-        <v>69908</v>
-      </c>
-      <c r="D8">
-        <v>179712</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B9" t="s">
-        <v>191</v>
-      </c>
-      <c r="C9">
-        <v>68978</v>
-      </c>
-      <c r="D9">
-        <v>179645</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B10" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10">
-        <v>70201</v>
-      </c>
-      <c r="D10">
-        <v>179653</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11">
-        <v>70088</v>
-      </c>
-      <c r="D11">
-        <v>179713</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C12">
-        <v>69737</v>
-      </c>
-      <c r="D12">
-        <v>179728</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B13" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13">
-        <v>67824</v>
-      </c>
-      <c r="D13">
-        <v>179694</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14">
-        <v>70390</v>
-      </c>
-      <c r="D14">
-        <v>179689</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B15" t="s">
-        <v>0</v>
-      </c>
-      <c r="D15">
-        <v>179647</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B16" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16">
-        <v>68147</v>
-      </c>
-      <c r="D16">
-        <v>179695</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B17" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17">
-        <v>69469</v>
-      </c>
-      <c r="D17">
-        <v>179723</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B18" t="s">
-        <v>29</v>
-      </c>
-      <c r="C18">
-        <v>66980</v>
-      </c>
-      <c r="D18">
-        <v>176367</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B19" t="s">
-        <v>187</v>
-      </c>
-      <c r="C19">
-        <v>70197</v>
-      </c>
-      <c r="D19">
-        <v>179658</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B20" t="s">
-        <v>29</v>
-      </c>
-      <c r="C20">
-        <v>69806</v>
-      </c>
-      <c r="D20">
-        <v>179657</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B21" t="s">
-        <v>86</v>
-      </c>
-      <c r="D21">
-        <v>179263</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B22" t="s">
-        <v>29</v>
-      </c>
-      <c r="C22">
-        <v>69802</v>
-      </c>
-      <c r="D22">
-        <v>179674</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C23">
-        <v>69767</v>
-      </c>
-      <c r="D23">
-        <v>179688</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B24" t="s">
-        <v>29</v>
-      </c>
-      <c r="C24">
-        <v>69814</v>
-      </c>
-      <c r="D24">
-        <v>179659</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B25" t="s">
-        <v>29</v>
-      </c>
-      <c r="D25">
-        <v>179707</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B26" t="s">
-        <v>29</v>
-      </c>
-      <c r="C26">
-        <v>69803</v>
-      </c>
-      <c r="D26">
-        <v>179671</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B27" t="s">
-        <v>86</v>
-      </c>
-      <c r="D27">
-        <v>179703</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B28" t="s">
-        <v>117</v>
-      </c>
-      <c r="D28">
-        <v>179679</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B29" t="s">
-        <v>29</v>
-      </c>
-      <c r="C29">
-        <v>70192</v>
-      </c>
-      <c r="D29">
-        <v>179716</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B30" t="s">
-        <v>117</v>
-      </c>
-      <c r="C30">
-        <v>70157</v>
-      </c>
-      <c r="D30">
-        <v>179690</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B31" t="s">
-        <v>86</v>
-      </c>
-      <c r="C31">
-        <v>69757</v>
-      </c>
-      <c r="D31">
-        <v>179638</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B32" t="s">
-        <v>117</v>
-      </c>
-      <c r="C32">
-        <v>69764</v>
-      </c>
-      <c r="D32">
-        <v>179650</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B33" t="s">
-        <v>29</v>
-      </c>
-      <c r="C33">
-        <v>70288</v>
-      </c>
-      <c r="D33">
-        <v>179655</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B34" t="s">
-        <v>187</v>
-      </c>
-      <c r="C34">
-        <v>68888</v>
-      </c>
-      <c r="D34">
-        <v>179636</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B35" t="s">
-        <v>86</v>
-      </c>
-      <c r="C35">
-        <v>70160</v>
-      </c>
-      <c r="D35">
-        <v>179673</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B36" t="s">
-        <v>187</v>
-      </c>
-      <c r="C36">
-        <v>69391</v>
-      </c>
-      <c r="D36">
-        <v>179639</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B37" t="s">
-        <v>74</v>
-      </c>
-      <c r="C37">
-        <v>69768</v>
-      </c>
-      <c r="D37">
-        <v>179660</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B38" t="s">
-        <v>86</v>
-      </c>
-      <c r="D38">
-        <v>179702</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B39" t="s">
-        <v>118</v>
-      </c>
-      <c r="D39">
-        <v>179706</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B40" t="s">
-        <v>74</v>
-      </c>
-      <c r="C40">
-        <v>69769</v>
-      </c>
-      <c r="D40">
-        <v>179640</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B41" t="s">
-        <v>86</v>
-      </c>
-      <c r="C41">
-        <v>69369</v>
-      </c>
-      <c r="D41">
-        <v>179641</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B42" t="s">
-        <v>86</v>
-      </c>
-      <c r="C42">
-        <v>70154</v>
-      </c>
-      <c r="D42">
-        <v>179637</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B43" t="s">
-        <v>86</v>
-      </c>
-      <c r="C43">
-        <v>69756</v>
-      </c>
-      <c r="D43">
-        <v>179701</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B44" t="s">
-        <v>118</v>
-      </c>
-      <c r="C44">
-        <v>69762</v>
-      </c>
-      <c r="D44">
-        <v>179661</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B45" t="s">
-        <v>86</v>
-      </c>
-      <c r="C45">
-        <v>69754</v>
-      </c>
-      <c r="D45">
-        <v>179722</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B46" t="s">
-        <v>86</v>
-      </c>
-      <c r="C46">
-        <v>70153</v>
-      </c>
-      <c r="D46">
-        <v>179656</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B47" t="s">
-        <v>158</v>
-      </c>
-      <c r="C47">
-        <v>539</v>
-      </c>
-      <c r="D47">
-        <v>534</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B48" t="s">
-        <v>40</v>
-      </c>
-      <c r="C48">
-        <v>549</v>
-      </c>
-      <c r="D48">
-        <v>540</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B49" t="s">
-        <v>24</v>
-      </c>
-      <c r="C49">
-        <v>546</v>
-      </c>
-      <c r="D49">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B50" t="s">
-        <v>24</v>
-      </c>
-      <c r="C50">
-        <v>547</v>
-      </c>
-      <c r="D50">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B51" t="s">
-        <v>40</v>
-      </c>
-      <c r="C51">
-        <v>548</v>
-      </c>
-      <c r="D51">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B52" t="s">
-        <v>192</v>
-      </c>
-      <c r="C52">
-        <v>70163</v>
-      </c>
-      <c r="D52">
-        <v>179642</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B53" t="s">
-        <v>193</v>
-      </c>
-      <c r="C53">
-        <v>69943</v>
-      </c>
-      <c r="D53">
-        <v>179662</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B54" t="s">
-        <v>166</v>
-      </c>
-      <c r="C54">
-        <v>69738</v>
-      </c>
-      <c r="D54">
-        <v>179751</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B55" t="s">
-        <v>194</v>
-      </c>
-      <c r="C55">
-        <v>70464</v>
-      </c>
-      <c r="D55">
-        <v>179779</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A56" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B56" t="s">
-        <v>19</v>
-      </c>
-      <c r="C56">
-        <v>69704</v>
-      </c>
-      <c r="D56">
-        <v>179780</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A57" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B57" t="s">
-        <v>7</v>
-      </c>
-      <c r="C57">
-        <v>70076</v>
-      </c>
-      <c r="D57">
-        <v>179556</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A58" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B58" t="s">
-        <v>19</v>
-      </c>
-      <c r="C58">
-        <v>70128</v>
-      </c>
-      <c r="D58">
-        <v>179616</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A59" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B59" t="s">
-        <v>19</v>
-      </c>
-      <c r="C59">
-        <v>70321</v>
-      </c>
-      <c r="D59">
-        <v>179675</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A60" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B60" t="s">
-        <v>19</v>
-      </c>
-      <c r="C60">
-        <v>69389</v>
-      </c>
-      <c r="D60">
-        <v>179785</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A61" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B61" t="s">
-        <v>19</v>
-      </c>
-      <c r="C61">
-        <v>68822</v>
-      </c>
-      <c r="D61">
-        <v>179783</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A62" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B62" t="s">
-        <v>19</v>
-      </c>
-      <c r="C62">
-        <v>69687</v>
-      </c>
-      <c r="D62">
-        <v>179782</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A63" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B63" t="s">
-        <v>19</v>
-      </c>
-      <c r="C63">
-        <v>70241</v>
-      </c>
-      <c r="D63">
-        <v>179781</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A64" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B64" t="s">
-        <v>89</v>
-      </c>
-      <c r="C64">
-        <v>70072</v>
-      </c>
-      <c r="D64">
-        <v>179681</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A65" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B65" t="s">
-        <v>121</v>
-      </c>
-      <c r="C65">
-        <v>70144</v>
-      </c>
-      <c r="D65">
-        <v>179676</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A66" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B66" t="s">
-        <v>121</v>
-      </c>
-      <c r="C66">
-        <v>70203</v>
-      </c>
-      <c r="D66">
-        <v>179685</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A67" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B67" t="s">
-        <v>121</v>
-      </c>
-      <c r="C67">
-        <v>70236</v>
-      </c>
-      <c r="D67">
-        <v>179684</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A68" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B68" t="s">
-        <v>122</v>
-      </c>
-      <c r="C68">
-        <v>70235</v>
-      </c>
-      <c r="D68">
-        <v>179726</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A69" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B69" t="s">
-        <v>195</v>
-      </c>
-      <c r="C69">
-        <v>70078</v>
-      </c>
-      <c r="D69">
-        <v>179677</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A70" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B70" t="s">
-        <v>122</v>
-      </c>
-      <c r="C70">
-        <v>69839</v>
-      </c>
-      <c r="D70">
-        <v>179678</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A71" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B71" t="s">
-        <v>18</v>
-      </c>
-      <c r="D71">
-        <v>18624</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A72" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B72" t="s">
-        <v>196</v>
-      </c>
-      <c r="C72">
-        <v>16289</v>
-      </c>
-      <c r="D72">
-        <v>18608</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A73" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B73" t="s">
-        <v>196</v>
-      </c>
-      <c r="C73">
-        <v>16293</v>
-      </c>
-      <c r="D73">
-        <v>18612</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A74" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B74" t="s">
-        <v>15</v>
-      </c>
-      <c r="C74">
-        <v>16305</v>
-      </c>
-      <c r="D74">
-        <v>18625</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A75" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B75" t="s">
-        <v>197</v>
-      </c>
-      <c r="C75">
-        <v>16299</v>
-      </c>
-      <c r="D75">
-        <v>18616</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A76" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B76" t="s">
-        <v>15</v>
-      </c>
-      <c r="C76">
-        <v>16300</v>
-      </c>
-      <c r="D76">
-        <v>18621</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A77" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B77" t="s">
-        <v>197</v>
-      </c>
-      <c r="D77">
-        <v>18617</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A78" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B78" t="s">
-        <v>198</v>
-      </c>
-      <c r="C78">
-        <v>16291</v>
-      </c>
-      <c r="D78">
-        <v>18610</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A79" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B79" t="s">
-        <v>196</v>
-      </c>
-      <c r="C79">
-        <v>16292</v>
-      </c>
-      <c r="D79">
-        <v>18611</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A80" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B80" t="s">
-        <v>199</v>
-      </c>
-      <c r="C80">
-        <v>16288</v>
-      </c>
-      <c r="D80">
-        <v>18607</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A81" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B81" t="s">
-        <v>200</v>
-      </c>
-      <c r="C81">
-        <v>16306</v>
-      </c>
-      <c r="D81">
-        <v>18618</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A82" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B82" t="s">
-        <v>15</v>
-      </c>
-      <c r="C82">
-        <v>16302</v>
-      </c>
-      <c r="D82">
-        <v>18622</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A83" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B83" t="s">
-        <v>201</v>
-      </c>
-      <c r="C83">
-        <v>16272</v>
-      </c>
-      <c r="D83">
-        <v>18603</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A84" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B84" t="s">
-        <v>202</v>
-      </c>
-      <c r="C84">
-        <v>16246</v>
-      </c>
-      <c r="D84">
-        <v>18605</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A85" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B85" t="s">
-        <v>203</v>
-      </c>
-      <c r="C85">
-        <v>16295</v>
-      </c>
-      <c r="D85">
-        <v>18614</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A86" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B86" t="s">
-        <v>201</v>
-      </c>
-      <c r="C86">
-        <v>16273</v>
-      </c>
-      <c r="D86">
-        <v>18606</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A87" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B87" t="s">
-        <v>201</v>
-      </c>
-      <c r="C87">
-        <v>16274</v>
-      </c>
-      <c r="D87">
-        <v>18601</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A88" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B88" t="s">
-        <v>15</v>
-      </c>
-      <c r="C88">
-        <v>16294</v>
-      </c>
-      <c r="D88">
-        <v>18613</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A89" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B89" t="s">
-        <v>15</v>
-      </c>
-      <c r="C89">
-        <v>16296</v>
-      </c>
-      <c r="D89">
-        <v>18615</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A90" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B90" t="s">
-        <v>15</v>
-      </c>
-      <c r="C90">
-        <v>16297</v>
-      </c>
-      <c r="D90">
-        <v>18619</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A91" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B91" t="s">
-        <v>23</v>
-      </c>
-      <c r="C91">
-        <v>68823</v>
-      </c>
-      <c r="D91">
-        <v>179790</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A92" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B92" t="s">
-        <v>23</v>
-      </c>
-      <c r="D92">
-        <v>179596</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A93" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B93" t="s">
-        <v>33</v>
-      </c>
-      <c r="C93">
-        <v>70315</v>
-      </c>
-      <c r="D93">
-        <v>179798</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A94" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B94" t="s">
-        <v>69</v>
-      </c>
-      <c r="C94">
-        <v>70453</v>
-      </c>
-      <c r="D94">
-        <v>179753</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A95" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B95" t="s">
-        <v>15</v>
-      </c>
-      <c r="C95">
-        <v>69645</v>
-      </c>
-      <c r="D95">
-        <v>179604</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A96" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B96" t="s">
-        <v>204</v>
-      </c>
-      <c r="C96">
-        <v>69840</v>
-      </c>
-      <c r="D96">
-        <v>179602</v>
-      </c>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A97" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B97" t="s">
-        <v>205</v>
-      </c>
-      <c r="D97">
-        <v>179368</v>
-      </c>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A98" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B98" t="s">
-        <v>19</v>
-      </c>
-      <c r="D98">
-        <v>179643</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A99" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B99" t="s">
-        <v>206</v>
-      </c>
-      <c r="C99">
-        <v>69551</v>
-      </c>
-      <c r="D99">
-        <v>179635</v>
-      </c>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A100" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B100" t="s">
-        <v>19</v>
-      </c>
-      <c r="D100">
-        <v>179767</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A101" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B101" t="s">
-        <v>15</v>
-      </c>
-      <c r="C101">
-        <v>70012</v>
-      </c>
-      <c r="D101">
-        <v>179608</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A102" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B102" t="s">
-        <v>12</v>
-      </c>
-      <c r="C102">
-        <v>69420</v>
-      </c>
-      <c r="D102">
-        <v>179625</v>
-      </c>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A103" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B103" t="s">
-        <v>19</v>
-      </c>
-      <c r="C103">
-        <v>70456</v>
-      </c>
-      <c r="D103">
-        <v>179784</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A104" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B104" t="s">
-        <v>207</v>
-      </c>
-      <c r="C104">
-        <v>70215</v>
-      </c>
-      <c r="D104">
-        <v>179696</v>
-      </c>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A105" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B105" t="s">
-        <v>207</v>
-      </c>
-      <c r="C105">
-        <v>70326</v>
-      </c>
-      <c r="D105">
-        <v>179700</v>
-      </c>
-    </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A106" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B106" t="s">
-        <v>8</v>
-      </c>
-      <c r="C106">
-        <v>70406</v>
-      </c>
-      <c r="D106">
-        <v>179826</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A107" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B107" t="s">
-        <v>207</v>
-      </c>
-      <c r="C107">
-        <v>70329</v>
-      </c>
-      <c r="D107">
-        <v>179717</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A108" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B108" t="s">
-        <v>207</v>
-      </c>
-      <c r="C108">
-        <v>70324</v>
-      </c>
-      <c r="D108">
-        <v>179698</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A109" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B109" t="s">
-        <v>207</v>
-      </c>
-      <c r="C109">
-        <v>70328</v>
-      </c>
-      <c r="D109">
-        <v>179714</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A110" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B110" t="s">
-        <v>8</v>
-      </c>
-      <c r="C110">
-        <v>70411</v>
-      </c>
-      <c r="D110">
-        <v>179831</v>
-      </c>
-    </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A111" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B111" t="s">
-        <v>207</v>
-      </c>
-      <c r="C111">
-        <v>70330</v>
-      </c>
-      <c r="D111">
-        <v>179719</v>
-      </c>
-    </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A112" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B112" t="s">
-        <v>207</v>
-      </c>
-      <c r="C112">
-        <v>70325</v>
-      </c>
-      <c r="D112">
-        <v>179699</v>
-      </c>
-    </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A113" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B113" t="s">
-        <v>8</v>
-      </c>
-      <c r="C113">
-        <v>70396</v>
-      </c>
-      <c r="D113">
-        <v>179787</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A114" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B114" t="s">
-        <v>8</v>
-      </c>
-      <c r="C114">
-        <v>70414</v>
-      </c>
-      <c r="D114">
-        <v>179834</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A115" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B115" t="s">
-        <v>8</v>
-      </c>
-      <c r="C115">
-        <v>70400</v>
-      </c>
-      <c r="D115">
-        <v>179819</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A116" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B116" t="s">
-        <v>207</v>
-      </c>
-      <c r="C116">
-        <v>70327</v>
-      </c>
-      <c r="D116">
-        <v>179709</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A117" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B117" t="s">
-        <v>11</v>
-      </c>
-      <c r="C117">
-        <v>70419</v>
-      </c>
-      <c r="D117">
-        <v>179841</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A118" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B118" t="s">
-        <v>8</v>
-      </c>
-      <c r="C118">
-        <v>70416</v>
-      </c>
-      <c r="D118">
-        <v>179836</v>
-      </c>
-    </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A119" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B119" t="s">
-        <v>8</v>
-      </c>
-      <c r="C119">
-        <v>70415</v>
-      </c>
-      <c r="D119">
-        <v>179835</v>
-      </c>
-    </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A120" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B120" t="s">
-        <v>8</v>
-      </c>
-      <c r="C120">
-        <v>70423</v>
-      </c>
-      <c r="D120">
-        <v>179845</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A121" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B121" t="s">
-        <v>11</v>
-      </c>
-      <c r="C121">
-        <v>70421</v>
-      </c>
-      <c r="D121">
-        <v>179838</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A122" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B122" t="s">
-        <v>8</v>
-      </c>
-      <c r="C122">
-        <v>70417</v>
-      </c>
-      <c r="D122">
-        <v>179837</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A123" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B123" t="s">
-        <v>11</v>
-      </c>
-      <c r="C123">
-        <v>70399</v>
-      </c>
-      <c r="D123">
-        <v>179810</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A124" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B124" t="s">
-        <v>11</v>
-      </c>
-      <c r="C124">
-        <v>70348</v>
-      </c>
-      <c r="D124">
-        <v>179774</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A125" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B125" t="s">
-        <v>11</v>
-      </c>
-      <c r="C125">
-        <v>70422</v>
-      </c>
-      <c r="D125">
-        <v>179843</v>
-      </c>
-    </row>
-    <row r="126" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A126" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B126" t="s">
-        <v>8</v>
-      </c>
-      <c r="C126">
-        <v>70431</v>
-      </c>
-      <c r="D126">
-        <v>179861</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A127" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B127" t="s">
-        <v>11</v>
-      </c>
-      <c r="C127">
-        <v>70436</v>
-      </c>
-      <c r="D127">
-        <v>179839</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A128" s="1">
-        <v>46315</v>
-      </c>
-      <c r="B128" t="s">
-        <v>11</v>
-      </c>
-      <c r="C128">
-        <v>70334</v>
-      </c>
-      <c r="D128">
-        <v>179732</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:D128" xr:uid="{3CCA1778-A08A-4BBC-894B-FE6DC9B4E104}"/>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualização dos dados dos KPIs
</commit_message>
<xml_diff>
--- a/DadosRomaneios.xlsx
+++ b/DadosRomaneios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1320ED70-5104-45CE-8E00-A8C7073D0C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7324FDFC-D845-40F9-A46A-88EADD39320A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1232" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1240" uniqueCount="233">
   <si>
     <t>ALBERT EINSTEIN</t>
   </si>
@@ -1140,7 +1140,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF29A37F-A1D1-4315-91AB-A952895E1E73}">
-  <dimension ref="A1:E1227"/>
+  <dimension ref="A1:E1235"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -21605,6 +21605,139 @@
       </c>
       <c r="E1227">
         <v>180059</v>
+      </c>
+    </row>
+    <row r="1228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1228" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1228">
+        <v>106</v>
+      </c>
+      <c r="C1228" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1228">
+        <v>574</v>
+      </c>
+      <c r="E1228">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="1229" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1229" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1229">
+        <v>106</v>
+      </c>
+      <c r="C1229" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1229">
+        <v>575</v>
+      </c>
+      <c r="E1229">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="1230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1230" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1230">
+        <v>101</v>
+      </c>
+      <c r="C1230" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1230">
+        <v>70452</v>
+      </c>
+      <c r="E1230">
+        <v>180125</v>
+      </c>
+    </row>
+    <row r="1231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1231" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1231">
+        <v>106</v>
+      </c>
+      <c r="C1231" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1231">
+        <v>580</v>
+      </c>
+      <c r="E1231">
+        <v>564</v>
+      </c>
+    </row>
+    <row r="1232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1232" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1232">
+        <v>106</v>
+      </c>
+      <c r="C1232" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1232">
+        <v>579</v>
+      </c>
+      <c r="E1232">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="1233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1233" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1233">
+        <v>101</v>
+      </c>
+      <c r="C1233" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1233">
+        <v>70200</v>
+      </c>
+      <c r="E1233">
+        <v>180126</v>
+      </c>
+    </row>
+    <row r="1234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1234" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1234">
+        <v>101</v>
+      </c>
+      <c r="C1234" t="s">
+        <v>15</v>
+      </c>
+      <c r="E1234">
+        <v>179651</v>
+      </c>
+    </row>
+    <row r="1235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1235" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B1235">
+        <v>101</v>
+      </c>
+      <c r="C1235" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1235">
+        <v>70781</v>
+      </c>
+      <c r="E1235">
+        <v>180167</v>
       </c>
     </row>
   </sheetData>
@@ -21785,7 +21918,7 @@
       </c>
       <c r="B18">
         <f>COUNTIF(Romaneios!A:A,DadosRomaneios!A18)</f>
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correção de dados errados
</commit_message>
<xml_diff>
--- a/DadosRomaneios.xlsx
+++ b/DadosRomaneios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E0D5981-269A-4404-8894-3C77D6C672D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AC4D3DC-196D-415A-A52C-DE045F23E809}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{B6976704-8E51-4052-B60A-5847F95A5AE5}"/>
   </bookViews>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1700" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1636" uniqueCount="264">
   <si>
     <t>ALBERT EINSTEIN</t>
   </si>
@@ -845,36 +845,6 @@
     <t>SYNGENTA PROTECAO</t>
   </si>
   <si>
-    <t>TEA RIBEIRAO PRETO</t>
-  </si>
-  <si>
-    <t>HOSP RIBEIRAO PRETO</t>
-  </si>
-  <si>
-    <t>DIAG ALTO BOA VISTA</t>
-  </si>
-  <si>
-    <t>CC RIBEIRAO PRETO</t>
-  </si>
-  <si>
-    <t>HAPCLINICA CAPIVARI</t>
-  </si>
-  <si>
-    <t>DIAG NACOES UNIDAS</t>
-  </si>
-  <si>
-    <t>CLINICA IRACEMAPOLIS</t>
-  </si>
-  <si>
-    <t>CLINICA SERRANA</t>
-  </si>
-  <si>
-    <t>CLINICA MORRO AGUDO</t>
-  </si>
-  <si>
-    <t>CLINICA PIRASSUNUNGA</t>
-  </si>
-  <si>
     <t>CONGREGACAO</t>
   </si>
   <si>
@@ -1264,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF29A37F-A1D1-4315-91AB-A952895E1E73}">
-  <dimension ref="A1:E1695"/>
+  <dimension ref="A1:E1631"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -27419,41 +27389,41 @@
     </row>
     <row r="1569" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1569" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1569">
         <v>101</v>
       </c>
       <c r="C1569" t="s">
-        <v>191</v>
+        <v>29</v>
       </c>
       <c r="D1569">
-        <v>69169</v>
+        <v>69980</v>
       </c>
       <c r="E1569">
-        <v>178863</v>
+        <v>180433</v>
       </c>
     </row>
     <row r="1570" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1570" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1570">
         <v>101</v>
       </c>
       <c r="C1570" t="s">
-        <v>39</v>
+        <v>85</v>
       </c>
       <c r="D1570">
-        <v>68863</v>
+        <v>70658</v>
       </c>
       <c r="E1570">
-        <v>178667</v>
+        <v>180640</v>
       </c>
     </row>
     <row r="1571" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1571" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1571">
         <v>101</v>
@@ -27462,100 +27432,97 @@
         <v>0</v>
       </c>
       <c r="D1571">
-        <v>69160</v>
+        <v>70889</v>
       </c>
       <c r="E1571">
-        <v>178631</v>
+        <v>180662</v>
       </c>
     </row>
     <row r="1572" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1572" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1572">
         <v>101</v>
       </c>
       <c r="C1572" t="s">
-        <v>260</v>
+        <v>0</v>
       </c>
       <c r="D1572">
-        <v>69509</v>
+        <v>70833</v>
       </c>
       <c r="E1572">
-        <v>178708</v>
+        <v>180468</v>
       </c>
     </row>
     <row r="1573" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1573" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1573">
         <v>101</v>
       </c>
       <c r="C1573" t="s">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="D1573">
-        <v>69911</v>
+        <v>69398</v>
       </c>
       <c r="E1573">
-        <v>179002</v>
+        <v>179106</v>
       </c>
     </row>
     <row r="1574" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1574" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1574">
         <v>101</v>
       </c>
       <c r="C1574" t="s">
-        <v>261</v>
+        <v>0</v>
       </c>
       <c r="D1574">
-        <v>69516</v>
+        <v>70107</v>
       </c>
       <c r="E1574">
-        <v>178709</v>
+        <v>180251</v>
       </c>
     </row>
     <row r="1575" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1575" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1575">
         <v>101</v>
       </c>
       <c r="C1575" t="s">
-        <v>262</v>
+        <v>0</v>
       </c>
       <c r="D1575">
-        <v>69506</v>
+        <v>70669</v>
       </c>
       <c r="E1575">
-        <v>178706</v>
+        <v>180267</v>
       </c>
     </row>
     <row r="1576" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1576" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1576">
         <v>101</v>
       </c>
       <c r="C1576" t="s">
-        <v>229</v>
-      </c>
-      <c r="D1576">
-        <v>69681</v>
+        <v>0</v>
       </c>
       <c r="E1576">
-        <v>178765</v>
+        <v>180430</v>
       </c>
     </row>
     <row r="1577" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1577" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1577">
         <v>101</v>
@@ -27564,66 +27531,66 @@
         <v>0</v>
       </c>
       <c r="D1577">
-        <v>69494</v>
+        <v>70834</v>
       </c>
       <c r="E1577">
-        <v>179063</v>
+        <v>180395</v>
       </c>
     </row>
     <row r="1578" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1578" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1578">
         <v>101</v>
       </c>
       <c r="C1578" t="s">
-        <v>263</v>
+        <v>0</v>
       </c>
       <c r="D1578">
-        <v>69507</v>
+        <v>69900</v>
       </c>
       <c r="E1578">
-        <v>178707</v>
+        <v>180396</v>
       </c>
     </row>
     <row r="1579" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1579" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1579">
         <v>101</v>
       </c>
       <c r="C1579" t="s">
-        <v>264</v>
+        <v>0</v>
       </c>
       <c r="D1579">
-        <v>69523</v>
+        <v>70822</v>
       </c>
       <c r="E1579">
-        <v>178710</v>
+        <v>180432</v>
       </c>
     </row>
     <row r="1580" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1580" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1580">
         <v>101</v>
       </c>
       <c r="C1580" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D1580">
-        <v>69404</v>
+        <v>70268</v>
       </c>
       <c r="E1580">
-        <v>179115</v>
+        <v>180589</v>
       </c>
     </row>
     <row r="1581" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1581" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1581">
         <v>101</v>
@@ -27632,134 +27599,131 @@
         <v>0</v>
       </c>
       <c r="D1581">
-        <v>69453</v>
+        <v>70106</v>
       </c>
       <c r="E1581">
-        <v>179319</v>
+        <v>180660</v>
       </c>
     </row>
     <row r="1582" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1582" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1582">
         <v>101</v>
       </c>
       <c r="C1582" t="s">
-        <v>191</v>
+        <v>260</v>
       </c>
       <c r="D1582">
-        <v>68977</v>
+        <v>71046</v>
       </c>
       <c r="E1582">
-        <v>178862</v>
+        <v>180656</v>
       </c>
     </row>
     <row r="1583" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1583" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1583">
         <v>101</v>
       </c>
       <c r="C1583" t="s">
-        <v>265</v>
+        <v>20</v>
       </c>
       <c r="D1583">
-        <v>69525</v>
+        <v>69037</v>
       </c>
       <c r="E1583">
-        <v>178705</v>
+        <v>180477</v>
       </c>
     </row>
     <row r="1584" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1584" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1584">
         <v>101</v>
       </c>
       <c r="C1584" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1584">
-        <v>69431</v>
+        <v>20</v>
       </c>
       <c r="E1584">
-        <v>179317</v>
+        <v>180626</v>
       </c>
     </row>
     <row r="1585" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1585" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1585">
         <v>101</v>
       </c>
       <c r="C1585" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="D1585">
-        <v>69532</v>
+        <v>70249</v>
       </c>
       <c r="E1585">
-        <v>179325</v>
+        <v>180597</v>
       </c>
     </row>
     <row r="1586" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1586" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1586">
         <v>101</v>
       </c>
       <c r="C1586" t="s">
-        <v>204</v>
+        <v>0</v>
       </c>
       <c r="D1586">
-        <v>69651</v>
+        <v>70178</v>
       </c>
       <c r="E1586">
-        <v>179046</v>
+        <v>180623</v>
       </c>
     </row>
     <row r="1587" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1587" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1587">
         <v>101</v>
       </c>
       <c r="C1587" t="s">
-        <v>158</v>
+        <v>45</v>
       </c>
       <c r="D1587">
-        <v>69613</v>
+        <v>69746</v>
       </c>
       <c r="E1587">
-        <v>178877</v>
+        <v>180637</v>
       </c>
     </row>
     <row r="1588" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1588" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1588">
         <v>101</v>
       </c>
       <c r="C1588" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="D1588">
-        <v>69922</v>
+        <v>69914</v>
       </c>
       <c r="E1588">
-        <v>179451</v>
+        <v>180650</v>
       </c>
     </row>
     <row r="1589" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1589" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1589">
         <v>101</v>
@@ -27767,16 +27731,13 @@
       <c r="C1589" t="s">
         <v>0</v>
       </c>
-      <c r="D1589">
-        <v>69864</v>
-      </c>
       <c r="E1589">
-        <v>179302</v>
+        <v>180570</v>
       </c>
     </row>
     <row r="1590" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1590" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1590">
         <v>101</v>
@@ -27785,15 +27746,15 @@
         <v>0</v>
       </c>
       <c r="D1590">
-        <v>69433</v>
+        <v>70493</v>
       </c>
       <c r="E1590">
-        <v>179304</v>
+        <v>180625</v>
       </c>
     </row>
     <row r="1591" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1591" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1591">
         <v>101</v>
@@ -27801,197 +27762,197 @@
       <c r="C1591" t="s">
         <v>0</v>
       </c>
-      <c r="D1591">
-        <v>69419</v>
-      </c>
       <c r="E1591">
-        <v>179064</v>
+        <v>180571</v>
       </c>
     </row>
     <row r="1592" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1592" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1592">
         <v>101</v>
       </c>
       <c r="C1592" t="s">
-        <v>266</v>
+        <v>113</v>
       </c>
       <c r="D1592">
-        <v>69919</v>
+        <v>69717</v>
       </c>
       <c r="E1592">
-        <v>179450</v>
+        <v>180574</v>
       </c>
     </row>
     <row r="1593" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1593" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1593">
         <v>101</v>
       </c>
       <c r="C1593" t="s">
-        <v>0</v>
+        <v>180</v>
       </c>
       <c r="D1593">
-        <v>70032</v>
+        <v>70492</v>
       </c>
       <c r="E1593">
-        <v>179341</v>
+        <v>180631</v>
       </c>
     </row>
     <row r="1594" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1594" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1594">
         <v>101</v>
       </c>
       <c r="C1594" t="s">
-        <v>0</v>
+        <v>111</v>
       </c>
       <c r="D1594">
-        <v>69890</v>
+        <v>69304</v>
       </c>
       <c r="E1594">
-        <v>179308</v>
+        <v>180629</v>
       </c>
     </row>
     <row r="1595" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1595" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1595">
         <v>101</v>
       </c>
       <c r="C1595" t="s">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="D1595">
-        <v>69728</v>
+        <v>70933</v>
       </c>
       <c r="E1595">
-        <v>179299</v>
+        <v>180635</v>
       </c>
     </row>
     <row r="1596" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1596" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1596">
         <v>101</v>
       </c>
       <c r="C1596" t="s">
-        <v>267</v>
+        <v>180</v>
       </c>
       <c r="D1596">
-        <v>70136</v>
+        <v>70230</v>
       </c>
       <c r="E1596">
-        <v>179447</v>
+        <v>180582</v>
       </c>
     </row>
     <row r="1597" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1597" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1597">
         <v>101</v>
       </c>
       <c r="C1597" t="s">
-        <v>268</v>
+        <v>45</v>
       </c>
       <c r="D1597">
-        <v>70145</v>
+        <v>70382</v>
       </c>
       <c r="E1597">
-        <v>179454</v>
+        <v>180652</v>
       </c>
     </row>
     <row r="1598" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1598" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1598">
         <v>101</v>
       </c>
       <c r="C1598" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1598">
-        <v>69902</v>
+        <v>60</v>
       </c>
       <c r="E1598">
-        <v>179366</v>
+        <v>180648</v>
       </c>
     </row>
     <row r="1599" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1599" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1599">
         <v>101</v>
       </c>
       <c r="C1599" t="s">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="D1599">
-        <v>69916</v>
+        <v>70490</v>
       </c>
       <c r="E1599">
-        <v>179449</v>
+        <v>180567</v>
       </c>
     </row>
     <row r="1600" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1600" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1600">
         <v>101</v>
       </c>
       <c r="C1600" t="s">
-        <v>0</v>
+        <v>60</v>
+      </c>
+      <c r="D1600">
+        <v>70067</v>
       </c>
       <c r="E1600">
-        <v>179758</v>
+        <v>180586</v>
       </c>
     </row>
     <row r="1601" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1601" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1601">
         <v>101</v>
       </c>
       <c r="C1601" t="s">
-        <v>7</v>
+        <v>256</v>
       </c>
       <c r="D1601">
-        <v>70091</v>
+        <v>70882</v>
       </c>
       <c r="E1601">
-        <v>179487</v>
+        <v>180392</v>
       </c>
     </row>
     <row r="1602" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1602" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1602">
         <v>101</v>
       </c>
       <c r="C1602" t="s">
-        <v>39</v>
+        <v>60</v>
+      </c>
+      <c r="D1602">
+        <v>70699</v>
       </c>
       <c r="E1602">
-        <v>179884</v>
+        <v>180585</v>
       </c>
     </row>
     <row r="1603" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1603" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1603">
         <v>101</v>
@@ -27999,44 +27960,50 @@
       <c r="C1603" t="s">
         <v>0</v>
       </c>
+      <c r="D1603">
+        <v>70025</v>
+      </c>
       <c r="E1603">
-        <v>179559</v>
+        <v>180573</v>
       </c>
     </row>
     <row r="1604" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1604" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1604">
         <v>101</v>
       </c>
       <c r="C1604" t="s">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="D1604">
+        <v>71038</v>
       </c>
       <c r="E1604">
-        <v>179815</v>
+        <v>180617</v>
       </c>
     </row>
     <row r="1605" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1605" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1605">
         <v>101</v>
       </c>
       <c r="C1605" t="s">
-        <v>183</v>
+        <v>0</v>
       </c>
       <c r="D1605">
-        <v>69361</v>
+        <v>70105</v>
       </c>
       <c r="E1605">
-        <v>179595</v>
+        <v>180624</v>
       </c>
     </row>
     <row r="1606" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1606" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1606">
         <v>101</v>
@@ -28045,1462 +28012,401 @@
         <v>0</v>
       </c>
       <c r="E1606">
-        <v>179804</v>
+        <v>180569</v>
       </c>
     </row>
     <row r="1607" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1607" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1607">
         <v>101</v>
       </c>
       <c r="C1607" t="s">
-        <v>269</v>
+        <v>167</v>
       </c>
       <c r="D1607">
-        <v>70318</v>
+        <v>69573</v>
       </c>
       <c r="E1607">
-        <v>179633</v>
+        <v>180638</v>
       </c>
     </row>
     <row r="1608" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1608" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1608">
         <v>101</v>
       </c>
       <c r="C1608" t="s">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="D1608">
-        <v>70095</v>
+        <v>70910</v>
       </c>
       <c r="E1608">
-        <v>179761</v>
+        <v>180622</v>
       </c>
     </row>
     <row r="1609" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1609" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1609">
         <v>101</v>
       </c>
       <c r="C1609" t="s">
-        <v>0</v>
+        <v>23</v>
+      </c>
+      <c r="D1609">
+        <v>69572</v>
       </c>
       <c r="E1609">
-        <v>179814</v>
+        <v>180627</v>
       </c>
     </row>
     <row r="1610" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1610" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1610">
         <v>101</v>
       </c>
       <c r="C1610" t="s">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D1610">
-        <v>69725</v>
+        <v>69824</v>
       </c>
       <c r="E1610">
-        <v>179867</v>
+        <v>180566</v>
       </c>
     </row>
     <row r="1611" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1611" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1611">
         <v>101</v>
       </c>
       <c r="C1611" t="s">
-        <v>183</v>
-      </c>
-      <c r="D1611">
-        <v>69362</v>
+        <v>33</v>
       </c>
       <c r="E1611">
-        <v>179598</v>
+        <v>180587</v>
       </c>
     </row>
     <row r="1612" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1612" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1612">
         <v>101</v>
       </c>
       <c r="C1612" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1612">
-        <v>70287</v>
+        <v>13</v>
       </c>
       <c r="E1612">
-        <v>179813</v>
+        <v>180599</v>
       </c>
     </row>
     <row r="1613" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1613" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1613">
         <v>101</v>
       </c>
       <c r="C1613" t="s">
-        <v>0</v>
+        <v>261</v>
       </c>
       <c r="D1613">
-        <v>69845</v>
+        <v>69788</v>
       </c>
       <c r="E1613">
-        <v>179868</v>
+        <v>180069</v>
       </c>
     </row>
     <row r="1614" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1614" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1614">
         <v>101</v>
       </c>
       <c r="C1614" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1614">
-        <v>69866</v>
+        <v>15</v>
       </c>
       <c r="E1614">
-        <v>179869</v>
+        <v>179394</v>
       </c>
     </row>
     <row r="1615" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1615" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1615">
         <v>101</v>
       </c>
       <c r="C1615" t="s">
-        <v>20</v>
+        <v>147</v>
       </c>
       <c r="D1615">
-        <v>70458</v>
+        <v>70552</v>
       </c>
       <c r="E1615">
-        <v>179729</v>
+        <v>180357</v>
       </c>
     </row>
     <row r="1616" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1616" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1616">
         <v>101</v>
       </c>
       <c r="C1616" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1616">
-        <v>70097</v>
+        <v>13</v>
       </c>
       <c r="E1616">
-        <v>179760</v>
+        <v>180643</v>
       </c>
     </row>
     <row r="1617" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1617" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1617">
         <v>101</v>
       </c>
       <c r="C1617" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="D1617">
-        <v>69882</v>
+        <v>69686</v>
       </c>
       <c r="E1617">
-        <v>179866</v>
+        <v>180600</v>
       </c>
     </row>
     <row r="1618" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1618" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1618">
         <v>101</v>
       </c>
       <c r="C1618" t="s">
-        <v>0</v>
+        <v>142</v>
       </c>
       <c r="D1618">
-        <v>70101</v>
+        <v>69791</v>
       </c>
       <c r="E1618">
-        <v>179811</v>
+        <v>180065</v>
       </c>
     </row>
     <row r="1619" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1619" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1619">
         <v>101</v>
       </c>
       <c r="C1619" t="s">
-        <v>0</v>
+        <v>262</v>
+      </c>
+      <c r="D1619">
+        <v>70557</v>
       </c>
       <c r="E1619">
-        <v>179764</v>
+        <v>180439</v>
       </c>
     </row>
     <row r="1620" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1620" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1620">
         <v>101</v>
       </c>
       <c r="C1620" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1620">
-        <v>70126</v>
+        <v>13</v>
       </c>
       <c r="E1620">
-        <v>179762</v>
+        <v>180655</v>
       </c>
     </row>
     <row r="1621" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1621" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1621">
         <v>101</v>
       </c>
       <c r="C1621" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="D1621">
-        <v>70098</v>
+        <v>70896</v>
       </c>
       <c r="E1621">
-        <v>179759</v>
+        <v>180654</v>
       </c>
     </row>
     <row r="1622" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1622" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1622">
         <v>101</v>
       </c>
       <c r="C1622" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="D1622">
-        <v>70179</v>
+        <v>70540</v>
       </c>
       <c r="E1622">
-        <v>179817</v>
+        <v>180591</v>
       </c>
     </row>
     <row r="1623" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1623" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1623">
         <v>101</v>
       </c>
       <c r="C1623" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E1623">
-        <v>179816</v>
+        <v>180658</v>
       </c>
     </row>
     <row r="1624" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1624" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1624">
         <v>101</v>
       </c>
       <c r="C1624" t="s">
-        <v>0</v>
+        <v>200</v>
       </c>
       <c r="D1624">
-        <v>70290</v>
+        <v>70912</v>
       </c>
       <c r="E1624">
-        <v>179809</v>
+        <v>180649</v>
       </c>
     </row>
     <row r="1625" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1625" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1625">
         <v>101</v>
       </c>
       <c r="C1625" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1625">
-        <v>69443</v>
+        <v>15</v>
       </c>
       <c r="E1625">
-        <v>180093</v>
+        <v>180601</v>
       </c>
     </row>
     <row r="1626" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1626" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1626">
         <v>101</v>
       </c>
       <c r="C1626" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1626">
-        <v>69698</v>
+        <v>13</v>
       </c>
       <c r="E1626">
-        <v>179993</v>
+        <v>180590</v>
       </c>
     </row>
     <row r="1627" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1627" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1627">
         <v>101</v>
       </c>
       <c r="C1627" t="s">
-        <v>0</v>
+        <v>89</v>
       </c>
       <c r="D1627">
-        <v>70100</v>
+        <v>70890</v>
       </c>
       <c r="E1627">
-        <v>179763</v>
+        <v>180651</v>
       </c>
     </row>
     <row r="1628" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1628" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1628">
         <v>101</v>
       </c>
       <c r="C1628" t="s">
-        <v>0</v>
+        <v>263</v>
       </c>
       <c r="D1628">
-        <v>70495</v>
+        <v>70554</v>
       </c>
       <c r="E1628">
-        <v>179994</v>
+        <v>180639</v>
       </c>
     </row>
     <row r="1629" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1629" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1629">
         <v>101</v>
       </c>
       <c r="C1629" t="s">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="D1629">
-        <v>70124</v>
+        <v>70938</v>
       </c>
       <c r="E1629">
-        <v>179812</v>
+        <v>180592</v>
       </c>
     </row>
     <row r="1630" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1630" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1630">
         <v>101</v>
       </c>
       <c r="C1630" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1630">
-        <v>70222</v>
+        <v>13</v>
       </c>
       <c r="E1630">
-        <v>179806</v>
+        <v>180593</v>
       </c>
     </row>
     <row r="1631" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1631" s="1">
-        <v>46323</v>
+        <v>46324</v>
       </c>
       <c r="B1631">
         <v>101</v>
       </c>
       <c r="C1631" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1631">
-        <v>70224</v>
+        <v>148</v>
       </c>
       <c r="E1631">
-        <v>179805</v>
-      </c>
-    </row>
-    <row r="1632" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1632" s="1">
-        <v>46323</v>
-      </c>
-      <c r="B1632">
-        <v>101</v>
-      </c>
-      <c r="C1632" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1632">
-        <v>69849</v>
-      </c>
-      <c r="E1632">
-        <v>180010</v>
-      </c>
-    </row>
-    <row r="1633" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1633" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1633">
-        <v>101</v>
-      </c>
-      <c r="C1633" t="s">
-        <v>29</v>
-      </c>
-      <c r="D1633">
-        <v>69980</v>
-      </c>
-      <c r="E1633">
-        <v>180433</v>
-      </c>
-    </row>
-    <row r="1634" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1634" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1634">
-        <v>101</v>
-      </c>
-      <c r="C1634" t="s">
-        <v>85</v>
-      </c>
-      <c r="D1634">
-        <v>70658</v>
-      </c>
-      <c r="E1634">
-        <v>180640</v>
-      </c>
-    </row>
-    <row r="1635" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1635" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1635">
-        <v>101</v>
-      </c>
-      <c r="C1635" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1635">
-        <v>70889</v>
-      </c>
-      <c r="E1635">
-        <v>180662</v>
-      </c>
-    </row>
-    <row r="1636" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1636" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1636">
-        <v>101</v>
-      </c>
-      <c r="C1636" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1636">
-        <v>70833</v>
-      </c>
-      <c r="E1636">
-        <v>180468</v>
-      </c>
-    </row>
-    <row r="1637" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1637" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1637">
-        <v>101</v>
-      </c>
-      <c r="C1637" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1637">
-        <v>69398</v>
-      </c>
-      <c r="E1637">
-        <v>179106</v>
-      </c>
-    </row>
-    <row r="1638" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1638" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1638">
-        <v>101</v>
-      </c>
-      <c r="C1638" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1638">
-        <v>70107</v>
-      </c>
-      <c r="E1638">
-        <v>180251</v>
-      </c>
-    </row>
-    <row r="1639" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1639" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1639">
-        <v>101</v>
-      </c>
-      <c r="C1639" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1639">
-        <v>70669</v>
-      </c>
-      <c r="E1639">
-        <v>180267</v>
-      </c>
-    </row>
-    <row r="1640" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1640" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1640">
-        <v>101</v>
-      </c>
-      <c r="C1640" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1640">
-        <v>180430</v>
-      </c>
-    </row>
-    <row r="1641" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1641" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1641">
-        <v>101</v>
-      </c>
-      <c r="C1641" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1641">
-        <v>70834</v>
-      </c>
-      <c r="E1641">
-        <v>180395</v>
-      </c>
-    </row>
-    <row r="1642" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1642" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1642">
-        <v>101</v>
-      </c>
-      <c r="C1642" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1642">
-        <v>69900</v>
-      </c>
-      <c r="E1642">
-        <v>180396</v>
-      </c>
-    </row>
-    <row r="1643" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1643" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1643">
-        <v>101</v>
-      </c>
-      <c r="C1643" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1643">
-        <v>70822</v>
-      </c>
-      <c r="E1643">
-        <v>180432</v>
-      </c>
-    </row>
-    <row r="1644" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1644" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1644">
-        <v>101</v>
-      </c>
-      <c r="C1644" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1644">
-        <v>70268</v>
-      </c>
-      <c r="E1644">
-        <v>180589</v>
-      </c>
-    </row>
-    <row r="1645" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1645" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1645">
-        <v>101</v>
-      </c>
-      <c r="C1645" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1645">
-        <v>70106</v>
-      </c>
-      <c r="E1645">
-        <v>180660</v>
-      </c>
-    </row>
-    <row r="1646" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1646" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1646">
-        <v>101</v>
-      </c>
-      <c r="C1646" t="s">
-        <v>270</v>
-      </c>
-      <c r="D1646">
-        <v>71046</v>
-      </c>
-      <c r="E1646">
-        <v>180656</v>
-      </c>
-    </row>
-    <row r="1647" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1647" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1647">
-        <v>101</v>
-      </c>
-      <c r="C1647" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1647">
-        <v>69037</v>
-      </c>
-      <c r="E1647">
-        <v>180477</v>
-      </c>
-    </row>
-    <row r="1648" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1648" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1648">
-        <v>101</v>
-      </c>
-      <c r="C1648" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1648">
-        <v>180626</v>
-      </c>
-    </row>
-    <row r="1649" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1649" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1649">
-        <v>101</v>
-      </c>
-      <c r="C1649" t="s">
-        <v>20</v>
-      </c>
-      <c r="D1649">
-        <v>70249</v>
-      </c>
-      <c r="E1649">
-        <v>180597</v>
-      </c>
-    </row>
-    <row r="1650" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1650" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1650">
-        <v>101</v>
-      </c>
-      <c r="C1650" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1650">
-        <v>70178</v>
-      </c>
-      <c r="E1650">
-        <v>180623</v>
-      </c>
-    </row>
-    <row r="1651" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1651" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1651">
-        <v>101</v>
-      </c>
-      <c r="C1651" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1651">
-        <v>69746</v>
-      </c>
-      <c r="E1651">
-        <v>180637</v>
-      </c>
-    </row>
-    <row r="1652" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1652" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1652">
-        <v>101</v>
-      </c>
-      <c r="C1652" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1652">
-        <v>69914</v>
-      </c>
-      <c r="E1652">
-        <v>180650</v>
-      </c>
-    </row>
-    <row r="1653" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1653" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1653">
-        <v>101</v>
-      </c>
-      <c r="C1653" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1653">
-        <v>180570</v>
-      </c>
-    </row>
-    <row r="1654" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1654" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1654">
-        <v>101</v>
-      </c>
-      <c r="C1654" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1654">
-        <v>70493</v>
-      </c>
-      <c r="E1654">
-        <v>180625</v>
-      </c>
-    </row>
-    <row r="1655" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1655" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1655">
-        <v>101</v>
-      </c>
-      <c r="C1655" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1655">
-        <v>180571</v>
-      </c>
-    </row>
-    <row r="1656" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1656" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1656">
-        <v>101</v>
-      </c>
-      <c r="C1656" t="s">
-        <v>113</v>
-      </c>
-      <c r="D1656">
-        <v>69717</v>
-      </c>
-      <c r="E1656">
-        <v>180574</v>
-      </c>
-    </row>
-    <row r="1657" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1657" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1657">
-        <v>101</v>
-      </c>
-      <c r="C1657" t="s">
-        <v>180</v>
-      </c>
-      <c r="D1657">
-        <v>70492</v>
-      </c>
-      <c r="E1657">
-        <v>180631</v>
-      </c>
-    </row>
-    <row r="1658" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1658" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1658">
-        <v>101</v>
-      </c>
-      <c r="C1658" t="s">
-        <v>111</v>
-      </c>
-      <c r="D1658">
-        <v>69304</v>
-      </c>
-      <c r="E1658">
-        <v>180629</v>
-      </c>
-    </row>
-    <row r="1659" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1659" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1659">
-        <v>101</v>
-      </c>
-      <c r="C1659" t="s">
-        <v>58</v>
-      </c>
-      <c r="D1659">
-        <v>70933</v>
-      </c>
-      <c r="E1659">
-        <v>180635</v>
-      </c>
-    </row>
-    <row r="1660" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1660" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1660">
-        <v>101</v>
-      </c>
-      <c r="C1660" t="s">
-        <v>180</v>
-      </c>
-      <c r="D1660">
-        <v>70230</v>
-      </c>
-      <c r="E1660">
-        <v>180582</v>
-      </c>
-    </row>
-    <row r="1661" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1661" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1661">
-        <v>101</v>
-      </c>
-      <c r="C1661" t="s">
-        <v>45</v>
-      </c>
-      <c r="D1661">
-        <v>70382</v>
-      </c>
-      <c r="E1661">
-        <v>180652</v>
-      </c>
-    </row>
-    <row r="1662" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1662" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1662">
-        <v>101</v>
-      </c>
-      <c r="C1662" t="s">
-        <v>60</v>
-      </c>
-      <c r="E1662">
-        <v>180648</v>
-      </c>
-    </row>
-    <row r="1663" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1663" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1663">
-        <v>101</v>
-      </c>
-      <c r="C1663" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1663">
-        <v>70490</v>
-      </c>
-      <c r="E1663">
-        <v>180567</v>
-      </c>
-    </row>
-    <row r="1664" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1664" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1664">
-        <v>101</v>
-      </c>
-      <c r="C1664" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1664">
-        <v>70067</v>
-      </c>
-      <c r="E1664">
-        <v>180586</v>
-      </c>
-    </row>
-    <row r="1665" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1665" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1665">
-        <v>101</v>
-      </c>
-      <c r="C1665" t="s">
-        <v>256</v>
-      </c>
-      <c r="D1665">
-        <v>70882</v>
-      </c>
-      <c r="E1665">
-        <v>180392</v>
-      </c>
-    </row>
-    <row r="1666" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1666" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1666">
-        <v>101</v>
-      </c>
-      <c r="C1666" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1666">
-        <v>70699</v>
-      </c>
-      <c r="E1666">
-        <v>180585</v>
-      </c>
-    </row>
-    <row r="1667" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1667" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1667">
-        <v>101</v>
-      </c>
-      <c r="C1667" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1667">
-        <v>70025</v>
-      </c>
-      <c r="E1667">
-        <v>180573</v>
-      </c>
-    </row>
-    <row r="1668" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1668" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1668">
-        <v>101</v>
-      </c>
-      <c r="C1668" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1668">
-        <v>71038</v>
-      </c>
-      <c r="E1668">
-        <v>180617</v>
-      </c>
-    </row>
-    <row r="1669" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1669" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1669">
-        <v>101</v>
-      </c>
-      <c r="C1669" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1669">
-        <v>70105</v>
-      </c>
-      <c r="E1669">
-        <v>180624</v>
-      </c>
-    </row>
-    <row r="1670" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1670" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1670">
-        <v>101</v>
-      </c>
-      <c r="C1670" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1670">
-        <v>180569</v>
-      </c>
-    </row>
-    <row r="1671" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1671" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1671">
-        <v>101</v>
-      </c>
-      <c r="C1671" t="s">
-        <v>167</v>
-      </c>
-      <c r="D1671">
-        <v>69573</v>
-      </c>
-      <c r="E1671">
-        <v>180638</v>
-      </c>
-    </row>
-    <row r="1672" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1672" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1672">
-        <v>101</v>
-      </c>
-      <c r="C1672" t="s">
-        <v>40</v>
-      </c>
-      <c r="D1672">
-        <v>70910</v>
-      </c>
-      <c r="E1672">
-        <v>180622</v>
-      </c>
-    </row>
-    <row r="1673" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1673" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1673">
-        <v>101</v>
-      </c>
-      <c r="C1673" t="s">
-        <v>23</v>
-      </c>
-      <c r="D1673">
-        <v>69572</v>
-      </c>
-      <c r="E1673">
-        <v>180627</v>
-      </c>
-    </row>
-    <row r="1674" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1674" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1674">
-        <v>101</v>
-      </c>
-      <c r="C1674" t="s">
-        <v>15</v>
-      </c>
-      <c r="D1674">
-        <v>69824</v>
-      </c>
-      <c r="E1674">
-        <v>180566</v>
-      </c>
-    </row>
-    <row r="1675" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1675" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1675">
-        <v>101</v>
-      </c>
-      <c r="C1675" t="s">
-        <v>33</v>
-      </c>
-      <c r="E1675">
-        <v>180587</v>
-      </c>
-    </row>
-    <row r="1676" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1676" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1676">
-        <v>101</v>
-      </c>
-      <c r="C1676" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1676">
-        <v>180599</v>
-      </c>
-    </row>
-    <row r="1677" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1677" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1677">
-        <v>101</v>
-      </c>
-      <c r="C1677" t="s">
-        <v>271</v>
-      </c>
-      <c r="D1677">
-        <v>69788</v>
-      </c>
-      <c r="E1677">
-        <v>180069</v>
-      </c>
-    </row>
-    <row r="1678" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1678" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1678">
-        <v>101</v>
-      </c>
-      <c r="C1678" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1678">
-        <v>179394</v>
-      </c>
-    </row>
-    <row r="1679" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1679" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1679">
-        <v>101</v>
-      </c>
-      <c r="C1679" t="s">
-        <v>147</v>
-      </c>
-      <c r="D1679">
-        <v>70552</v>
-      </c>
-      <c r="E1679">
-        <v>180357</v>
-      </c>
-    </row>
-    <row r="1680" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1680" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1680">
-        <v>101</v>
-      </c>
-      <c r="C1680" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1680">
-        <v>180643</v>
-      </c>
-    </row>
-    <row r="1681" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1681" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1681">
-        <v>101</v>
-      </c>
-      <c r="C1681" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1681">
-        <v>69686</v>
-      </c>
-      <c r="E1681">
-        <v>180600</v>
-      </c>
-    </row>
-    <row r="1682" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1682" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1682">
-        <v>101</v>
-      </c>
-      <c r="C1682" t="s">
-        <v>142</v>
-      </c>
-      <c r="D1682">
-        <v>69791</v>
-      </c>
-      <c r="E1682">
-        <v>180065</v>
-      </c>
-    </row>
-    <row r="1683" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1683" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1683">
-        <v>101</v>
-      </c>
-      <c r="C1683" t="s">
-        <v>272</v>
-      </c>
-      <c r="D1683">
-        <v>70557</v>
-      </c>
-      <c r="E1683">
-        <v>180439</v>
-      </c>
-    </row>
-    <row r="1684" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1684" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1684">
-        <v>101</v>
-      </c>
-      <c r="C1684" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1684">
-        <v>180655</v>
-      </c>
-    </row>
-    <row r="1685" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1685" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1685">
-        <v>101</v>
-      </c>
-      <c r="C1685" t="s">
-        <v>13</v>
-      </c>
-      <c r="D1685">
-        <v>70896</v>
-      </c>
-      <c r="E1685">
-        <v>180654</v>
-      </c>
-    </row>
-    <row r="1686" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1686" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1686">
-        <v>101</v>
-      </c>
-      <c r="C1686" t="s">
-        <v>16</v>
-      </c>
-      <c r="D1686">
-        <v>70540</v>
-      </c>
-      <c r="E1686">
-        <v>180591</v>
-      </c>
-    </row>
-    <row r="1687" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1687" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1687">
-        <v>101</v>
-      </c>
-      <c r="C1687" t="s">
-        <v>16</v>
-      </c>
-      <c r="E1687">
-        <v>180658</v>
-      </c>
-    </row>
-    <row r="1688" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1688" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1688">
-        <v>101</v>
-      </c>
-      <c r="C1688" t="s">
-        <v>200</v>
-      </c>
-      <c r="D1688">
-        <v>70912</v>
-      </c>
-      <c r="E1688">
-        <v>180649</v>
-      </c>
-    </row>
-    <row r="1689" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1689" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1689">
-        <v>101</v>
-      </c>
-      <c r="C1689" t="s">
-        <v>15</v>
-      </c>
-      <c r="E1689">
-        <v>180601</v>
-      </c>
-    </row>
-    <row r="1690" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1690" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1690">
-        <v>101</v>
-      </c>
-      <c r="C1690" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1690">
-        <v>180590</v>
-      </c>
-    </row>
-    <row r="1691" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1691" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1691">
-        <v>101</v>
-      </c>
-      <c r="C1691" t="s">
-        <v>89</v>
-      </c>
-      <c r="D1691">
-        <v>70890</v>
-      </c>
-      <c r="E1691">
-        <v>180651</v>
-      </c>
-    </row>
-    <row r="1692" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1692" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1692">
-        <v>101</v>
-      </c>
-      <c r="C1692" t="s">
-        <v>273</v>
-      </c>
-      <c r="D1692">
-        <v>70554</v>
-      </c>
-      <c r="E1692">
-        <v>180639</v>
-      </c>
-    </row>
-    <row r="1693" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1693" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1693">
-        <v>101</v>
-      </c>
-      <c r="C1693" t="s">
-        <v>147</v>
-      </c>
-      <c r="D1693">
-        <v>70938</v>
-      </c>
-      <c r="E1693">
-        <v>180592</v>
-      </c>
-    </row>
-    <row r="1694" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1694" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1694">
-        <v>101</v>
-      </c>
-      <c r="C1694" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1694">
-        <v>180593</v>
-      </c>
-    </row>
-    <row r="1695" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1695" s="1">
-        <v>46324</v>
-      </c>
-      <c r="B1695">
-        <v>101</v>
-      </c>
-      <c r="C1695" t="s">
-        <v>148</v>
-      </c>
-      <c r="E1695">
         <v>180641</v>
       </c>
     </row>
@@ -29727,7 +28633,7 @@
       </c>
       <c r="B22">
         <f>COUNTIF(Romaneios!A:A,DadosRomaneios!A22)</f>
-        <v>153</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>